<commit_message>
Fixed: - Bumped version to 1.1.0 - Moved HTML and JS files from core/ to assets/ - Outputting Sankey graphs to separate HTML files was improperly using os.path.join() instead of importlib.resources.files() - Removed comment-like columns from Process - Updated tests - Updated example_scenario.xlsx
</commit_message>
<xml_diff>
--- a/src/aiphoria/data/example_scenario.xlsx
+++ b/src/aiphoria/data/example_scenario.xlsx
@@ -1,31 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\PythonProjects\aiphoria\src\aiphoria\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B89CE2A-CFA9-4264-9CC9-BBBA7361EB5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9EAEAA4-B353-41EC-82AF-073964581B1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-25635" yWindow="2265" windowWidth="21600" windowHeight="11295" activeTab="5" xr2:uid="{1000A452-A98F-45C1-B843-91F7F67E097C}"/>
+    <workbookView xWindow="1620" yWindow="2175" windowWidth="21600" windowHeight="11295" xr2:uid="{1000A452-A98F-45C1-B843-91F7F67E097C}"/>
   </bookViews>
   <sheets>
-    <sheet name="Settings" sheetId="11" r:id="rId1"/>
-    <sheet name="Processes" sheetId="6" r:id="rId2"/>
-    <sheet name="Flows" sheetId="1" r:id="rId3"/>
-    <sheet name="Stock lifetime overrides" sheetId="15" r:id="rId4"/>
-    <sheet name="Process positions" sheetId="14" r:id="rId5"/>
-    <sheet name="Scenarios" sheetId="12" r:id="rId6"/>
-    <sheet name="Colors" sheetId="13" r:id="rId7"/>
-    <sheet name="Data validation parameters" sheetId="9" r:id="rId8"/>
+    <sheet name="INFO" sheetId="16" r:id="rId1"/>
+    <sheet name="Settings" sheetId="11" r:id="rId2"/>
+    <sheet name="Processes" sheetId="6" r:id="rId3"/>
+    <sheet name="Flows" sheetId="1" r:id="rId4"/>
+    <sheet name="Stock lifetime overrides" sheetId="15" r:id="rId5"/>
+    <sheet name="Process positions" sheetId="14" r:id="rId6"/>
+    <sheet name="Scenarios" sheetId="12" r:id="rId7"/>
+    <sheet name="Colors" sheetId="13" r:id="rId8"/>
+    <sheet name="Data validation parameters" sheetId="9" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Flows!$A$3:$P$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Processes!$D$3:$R$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Settings!$B$6:$E$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Flows!$A$3:$P$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Processes!$D$3:$R$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Settings!$B$6:$E$6</definedName>
     <definedName name="Boolean">'Data validation parameters'!$C$6:$C$7</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
@@ -49,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="524" uniqueCount="240">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="541" uniqueCount="252">
   <si>
     <t>Years</t>
   </si>
@@ -79,9 +80,6 @@
   </si>
   <si>
     <t>%</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> kg/m3</t>
   </si>
   <si>
     <t>Density</t>
@@ -813,6 +811,45 @@
   </si>
   <si>
     <t>prioritize_transformation_stages</t>
+  </si>
+  <si>
+    <t>% (Optional)</t>
+  </si>
+  <si>
+    <t>(Optional)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> kg/m3 (Optional)</t>
+  </si>
+  <si>
+    <t>This is aiphoria settings file</t>
+  </si>
+  <si>
+    <t>Refer to the aiphoria wiki for the detailed explanation of different sheets.</t>
+  </si>
+  <si>
+    <t>Green colored columns are comment / optional fields and could be left blank or removed.</t>
+  </si>
+  <si>
+    <t>Check what columns are defined as comment columns in Settings-sheet</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>A,G,J,K,L,M,N</t>
+  </si>
+  <si>
+    <t>A,M,N</t>
+  </si>
+  <si>
+    <t>This column is ignored (check parameter ignore_columns_scenarios in Settings-sheet)</t>
+  </si>
+  <si>
+    <t>skip_num_rows_scenarios</t>
+  </si>
+  <si>
+    <t>Number of rows to skip when reading data for Scenarios (e.g. 2). NOTE: Header row must be the first row to read!</t>
   </si>
 </sst>
 </file>
@@ -888,7 +925,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -904,6 +941,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFE7E6E6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -962,7 +1005,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -984,12 +1027,6 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -1002,7 +1039,22 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1464,8 +1516,41 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83DA9B50-109E-4569-8896-9B271C0F5058}">
+  <dimension ref="A2:B7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>246</v>
+      </c>
+      <c r="B7" t="s">
+        <v>245</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89FFA668-DA1A-459B-BD42-D0D7F7709F0D}">
-  <dimension ref="A2:E41"/>
+  <dimension ref="A2:E42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.7109375" bestFit="1" customWidth="1"/>
@@ -1476,32 +1561,32 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:5" ht="21" x14ac:dyDescent="0.35">
-      <c r="B2" s="19" t="s">
-        <v>62</v>
+      <c r="B2" s="17" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="3" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B3" s="21" t="s">
-        <v>81</v>
+      <c r="B3" s="19" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="4" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
-        <v>80</v>
-      </c>
-      <c r="C4" s="21"/>
-      <c r="D4" s="21"/>
-      <c r="E4" s="21"/>
+        <v>79</v>
+      </c>
+      <c r="C4" s="19"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
     </row>
     <row r="6" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B6" s="9" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E6" s="9" t="s">
         <v>3</v>
@@ -1509,430 +1594,433 @@
     </row>
     <row r="7" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
-        <v>64</v>
-      </c>
-      <c r="C7" s="23" t="s">
+        <v>63</v>
+      </c>
+      <c r="C7" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="23" t="s">
-        <v>92</v>
+      <c r="D7" s="21" t="s">
+        <v>91</v>
       </c>
       <c r="E7" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="8" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C8" t="s">
-        <v>182</v>
+        <v>247</v>
       </c>
       <c r="D8" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E8" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="9" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
-        <v>65</v>
-      </c>
-      <c r="C9" s="22">
+        <v>64</v>
+      </c>
+      <c r="C9" s="20">
         <v>2</v>
       </c>
-      <c r="D9" s="22" t="s">
-        <v>90</v>
+      <c r="D9" s="20" t="s">
+        <v>89</v>
       </c>
       <c r="E9" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="10" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
-        <v>66</v>
-      </c>
-      <c r="C10" s="23" t="s">
+        <v>65</v>
+      </c>
+      <c r="C10" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="D10" s="23" t="s">
-        <v>91</v>
+      <c r="D10" s="21" t="s">
+        <v>90</v>
       </c>
       <c r="E10" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="11" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C11" t="s">
-        <v>182</v>
+        <v>248</v>
       </c>
       <c r="D11" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E11" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="12" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
+        <v>66</v>
+      </c>
+      <c r="C12" s="20">
+        <v>2</v>
+      </c>
+      <c r="D12" s="20" t="s">
+        <v>89</v>
+      </c>
+      <c r="E12" t="s">
         <v>67</v>
-      </c>
-      <c r="C12" s="22">
-        <v>2</v>
-      </c>
-      <c r="D12" s="22" t="s">
-        <v>90</v>
-      </c>
-      <c r="E12" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="13" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
+        <v>68</v>
+      </c>
+      <c r="C13" s="20">
+        <v>2021</v>
+      </c>
+      <c r="D13" s="20" t="s">
+        <v>89</v>
+      </c>
+      <c r="E13" t="s">
         <v>69</v>
-      </c>
-      <c r="C13" s="22">
-        <v>2021</v>
-      </c>
-      <c r="D13" s="22" t="s">
-        <v>90</v>
-      </c>
-      <c r="E13" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="14" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
-        <v>71</v>
-      </c>
-      <c r="C14" s="22">
+        <v>70</v>
+      </c>
+      <c r="C14" s="20">
         <v>2030</v>
       </c>
-      <c r="D14" s="22" t="s">
-        <v>90</v>
+      <c r="D14" s="20" t="s">
+        <v>89</v>
       </c>
       <c r="E14" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="15" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
-        <v>72</v>
-      </c>
-      <c r="C15" s="24" t="b">
+        <v>71</v>
+      </c>
+      <c r="C15" s="22" t="b">
         <v>0</v>
       </c>
       <c r="D15" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E15" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="16" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
+        <v>74</v>
+      </c>
+      <c r="C16" s="22" t="b">
+        <v>1</v>
+      </c>
+      <c r="D16" t="s">
+        <v>88</v>
+      </c>
+      <c r="E16" t="s">
         <v>75</v>
-      </c>
-      <c r="C16" s="24" t="b">
-        <v>1</v>
-      </c>
-      <c r="D16" t="s">
-        <v>89</v>
-      </c>
-      <c r="E16" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C17" s="14">
         <v>0.1</v>
       </c>
-      <c r="D17" s="22" t="s">
-        <v>93</v>
+      <c r="D17" s="20" t="s">
+        <v>92</v>
       </c>
       <c r="E17" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B18" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C18" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D18" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E18" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B19" t="s">
+        <v>173</v>
+      </c>
+      <c r="C19" t="s">
+        <v>176</v>
+      </c>
+      <c r="D19" t="s">
+        <v>90</v>
+      </c>
+      <c r="E19" t="s">
         <v>174</v>
-      </c>
-      <c r="C19" t="s">
-        <v>177</v>
-      </c>
-      <c r="D19" t="s">
-        <v>91</v>
-      </c>
-      <c r="E19" t="s">
-        <v>175</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B20" t="s">
+        <v>76</v>
+      </c>
+      <c r="C20" s="18">
+        <v>-3.6666666666666701</v>
+      </c>
+      <c r="D20" s="18" t="s">
+        <v>92</v>
+      </c>
+      <c r="E20" t="s">
         <v>77</v>
-      </c>
-      <c r="C20" s="20">
-        <v>-3.6666666666666701</v>
-      </c>
-      <c r="D20" s="20" t="s">
-        <v>93</v>
-      </c>
-      <c r="E20" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B21" t="s">
+        <v>86</v>
+      </c>
+      <c r="C21" s="22" t="b">
+        <v>1</v>
+      </c>
+      <c r="D21" t="s">
+        <v>88</v>
+      </c>
+      <c r="E21" t="s">
         <v>87</v>
-      </c>
-      <c r="C21" s="24" t="b">
-        <v>1</v>
-      </c>
-      <c r="D21" t="s">
-        <v>89</v>
-      </c>
-      <c r="E21" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B22" t="s">
-        <v>86</v>
-      </c>
-      <c r="C22" s="24" t="b">
+        <v>85</v>
+      </c>
+      <c r="C22" s="22" t="b">
         <v>1</v>
       </c>
       <c r="D22" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E22" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B23" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C23" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D23" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E23" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B24" t="s">
+        <v>184</v>
+      </c>
+      <c r="C24" s="22" t="b">
+        <v>1</v>
+      </c>
+      <c r="D24" t="s">
+        <v>88</v>
+      </c>
+      <c r="E24" t="s">
         <v>185</v>
-      </c>
-      <c r="C24" s="24" t="b">
-        <v>1</v>
-      </c>
-      <c r="D24" t="s">
-        <v>89</v>
-      </c>
-      <c r="E24" t="s">
-        <v>186</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B25" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C25" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="D25" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E25" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B26" t="s">
+        <v>99</v>
+      </c>
+      <c r="C26" t="s">
         <v>100</v>
       </c>
-      <c r="C26" t="s">
-        <v>101</v>
-      </c>
       <c r="D26" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E26" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B27" t="s">
-        <v>161</v>
+        <v>160</v>
+      </c>
+      <c r="C27" t="s">
+        <v>181</v>
       </c>
       <c r="D27" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E27" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B28" t="s">
-        <v>102</v>
-      </c>
-      <c r="C28" s="24" t="b">
-        <v>1</v>
+        <v>250</v>
       </c>
       <c r="D28" t="s">
         <v>89</v>
       </c>
       <c r="E28" t="s">
-        <v>103</v>
+        <v>251</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B29" t="s">
-        <v>104</v>
-      </c>
-      <c r="C29" s="24" t="b">
+        <v>101</v>
+      </c>
+      <c r="C29" s="22" t="b">
         <v>1</v>
       </c>
       <c r="D29" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E29" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B30" t="s">
-        <v>123</v>
-      </c>
-      <c r="C30" t="s">
-        <v>126</v>
+        <v>103</v>
+      </c>
+      <c r="C30" s="22" t="b">
+        <v>1</v>
       </c>
       <c r="D30" t="s">
-        <v>125</v>
+        <v>88</v>
       </c>
       <c r="E30" t="s">
-        <v>124</v>
+        <v>104</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B31" t="s">
-        <v>143</v>
-      </c>
-      <c r="C31" s="22" t="s">
-        <v>144</v>
-      </c>
-      <c r="D31" s="22" t="s">
-        <v>91</v>
+        <v>122</v>
+      </c>
+      <c r="C31" t="s">
+        <v>125</v>
+      </c>
+      <c r="D31" t="s">
+        <v>124</v>
       </c>
       <c r="E31" t="s">
-        <v>235</v>
+        <v>123</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B32" t="s">
-        <v>162</v>
-      </c>
-      <c r="D32" t="s">
-        <v>125</v>
+        <v>142</v>
+      </c>
+      <c r="C32" s="20" t="s">
+        <v>143</v>
+      </c>
+      <c r="D32" s="20" t="s">
+        <v>90</v>
       </c>
       <c r="E32" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B33" t="s">
-        <v>188</v>
+        <v>161</v>
       </c>
       <c r="D33" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E33" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B34" t="s">
-        <v>239</v>
+        <v>187</v>
       </c>
       <c r="D34" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E34" t="s">
         <v>190</v>
@@ -1940,121 +2028,135 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B35" t="s">
-        <v>200</v>
-      </c>
-      <c r="C35" t="s">
-        <v>201</v>
+        <v>238</v>
       </c>
       <c r="D35" t="s">
-        <v>91</v>
+        <v>124</v>
       </c>
       <c r="E35" t="s">
-        <v>234</v>
+        <v>189</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
+        <v>198</v>
+      </c>
+      <c r="B36" t="s">
         <v>199</v>
       </c>
-      <c r="B36" t="s">
-        <v>210</v>
-      </c>
       <c r="C36" t="s">
-        <v>211</v>
+        <v>200</v>
       </c>
       <c r="D36" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E36" t="s">
-        <v>212</v>
+        <v>233</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B37" t="s">
-        <v>213</v>
-      </c>
-      <c r="C37" s="24" t="b">
-        <v>1</v>
+        <v>209</v>
+      </c>
+      <c r="C37" t="s">
+        <v>210</v>
       </c>
       <c r="D37" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E37" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B38" t="s">
-        <v>225</v>
-      </c>
-      <c r="C38" s="24" t="b">
+        <v>212</v>
+      </c>
+      <c r="C38" s="22" t="b">
         <v>1</v>
       </c>
       <c r="D38" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E38" t="s">
-        <v>226</v>
+        <v>213</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B39" t="s">
-        <v>227</v>
-      </c>
-      <c r="C39" t="s">
-        <v>228</v>
+        <v>224</v>
+      </c>
+      <c r="C39" s="22" t="b">
+        <v>1</v>
       </c>
       <c r="D39" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="E39" t="s">
-        <v>233</v>
+        <v>225</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B40" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="C40" t="s">
-        <v>182</v>
+        <v>227</v>
       </c>
       <c r="D40" t="s">
-        <v>125</v>
+        <v>90</v>
       </c>
       <c r="E40" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B41" t="s">
+        <v>228</v>
+      </c>
+      <c r="C41" t="s">
+        <v>181</v>
+      </c>
+      <c r="D41" t="s">
+        <v>124</v>
+      </c>
+      <c r="E41" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>198</v>
+      </c>
+      <c r="B42" t="s">
+        <v>230</v>
+      </c>
+      <c r="C42">
+        <v>2</v>
+      </c>
+      <c r="D42" t="s">
+        <v>89</v>
+      </c>
+      <c r="E42" t="s">
         <v>231</v>
-      </c>
-      <c r="C41">
-        <v>2</v>
-      </c>
-      <c r="D41" t="s">
-        <v>90</v>
-      </c>
-      <c r="E41" t="s">
-        <v>232</v>
       </c>
     </row>
   </sheetData>
@@ -2083,7 +2185,7 @@
       <formula>TRUE</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C28:C29">
+  <conditionalFormatting sqref="C29:C30">
     <cfRule type="cellIs" dxfId="5" priority="7" operator="equal">
       <formula>TRUE</formula>
     </cfRule>
@@ -2091,7 +2193,7 @@
       <formula>TRUE</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C37:C38">
+  <conditionalFormatting sqref="C38:C39">
     <cfRule type="cellIs" dxfId="3" priority="3" operator="equal">
       <formula>TRUE</formula>
     </cfRule>
@@ -2100,7 +2202,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C15:C16 C21:C22 C28:C29 C24 C37:C38" xr:uid="{79A7E31C-3284-4405-9B5F-03E099B07563}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C15:C16 C21:C22 C29:C30 C24 C38:C39" xr:uid="{79A7E31C-3284-4405-9B5F-03E099B07563}">
       <formula1>Boolean</formula1>
     </dataValidation>
   </dataValidations>
@@ -2127,32 +2229,32 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32C0D592-75C1-4AD1-84F0-2AAE25CA0097}">
   <dimension ref="A1:R18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.7109375" customWidth="1"/>
+    <col min="1" max="1" width="24.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="21" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="23.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.5703125" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" customWidth="1"/>
-    <col min="7" max="7" width="17" customWidth="1"/>
-    <col min="8" max="8" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="25" customWidth="1"/>
-    <col min="10" max="10" width="17.42578125" customWidth="1"/>
-    <col min="11" max="11" width="24.5703125" customWidth="1"/>
-    <col min="12" max="12" width="9.85546875" customWidth="1"/>
-    <col min="13" max="13" width="18.28515625" customWidth="1"/>
-    <col min="14" max="14" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="22.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.5703125" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="9.7109375" bestFit="1" customWidth="1"/>
     <col min="16" max="17" width="12.85546875" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="19.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A1" s="1"/>
+      <c r="A1" s="27"/>
       <c r="B1" s="2" t="s">
         <v>5</v>
       </c>
@@ -2168,33 +2270,33 @@
       <c r="F1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="2"/>
+      <c r="G1" s="23"/>
       <c r="H1" s="2" t="s">
         <v>5</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="J1" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="J1" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" s="23" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="L1" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="M1" s="23" t="s">
         <v>5</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="N1" s="23" t="s">
         <v>5</v>
       </c>
       <c r="O1" s="2" t="s">
         <v>5</v>
       </c>
       <c r="P1" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="Q1" s="2" t="s">
         <v>7</v>
@@ -2204,7 +2306,7 @@
       </c>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A2" s="1"/>
+      <c r="A2" s="27"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
@@ -2212,77 +2314,85 @@
       <c r="F2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="G2" s="2"/>
+      <c r="G2" s="23" t="s">
+        <v>240</v>
+      </c>
       <c r="H2" s="2"/>
       <c r="I2" s="7"/>
-      <c r="J2" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="K2" s="2"/>
-      <c r="L2" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="M2" s="2"/>
-      <c r="N2" s="2"/>
+      <c r="J2" s="23" t="s">
+        <v>239</v>
+      </c>
+      <c r="K2" s="23" t="s">
+        <v>240</v>
+      </c>
+      <c r="L2" s="23" t="s">
+        <v>241</v>
+      </c>
+      <c r="M2" s="23" t="s">
+        <v>240</v>
+      </c>
+      <c r="N2" s="23" t="s">
+        <v>240</v>
+      </c>
       <c r="O2" s="2"/>
       <c r="P2" s="2"/>
       <c r="Q2" s="1"/>
       <c r="R2" s="1"/>
     </row>
-    <row r="3" spans="1:18" s="17" customFormat="1" ht="60" x14ac:dyDescent="0.25">
-      <c r="A3" s="15" t="s">
-        <v>183</v>
-      </c>
-      <c r="B3" s="16" t="s">
+    <row r="3" spans="1:18" s="15" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+      <c r="A3" s="28" t="s">
+        <v>182</v>
+      </c>
+      <c r="B3" s="29" t="s">
+        <v>58</v>
+      </c>
+      <c r="C3" s="29" t="s">
+        <v>153</v>
+      </c>
+      <c r="D3" s="29" t="s">
+        <v>41</v>
+      </c>
+      <c r="E3" s="29" t="s">
+        <v>154</v>
+      </c>
+      <c r="F3" s="29" t="s">
         <v>59</v>
       </c>
-      <c r="C3" s="16" t="s">
-        <v>154</v>
-      </c>
-      <c r="D3" s="16" t="s">
-        <v>42</v>
-      </c>
-      <c r="E3" s="16" t="s">
+      <c r="G3" s="24" t="s">
         <v>155</v>
       </c>
-      <c r="F3" s="16" t="s">
-        <v>60</v>
-      </c>
-      <c r="G3" s="16" t="s">
+      <c r="H3" s="29" t="s">
+        <v>84</v>
+      </c>
+      <c r="I3" s="29" t="s">
         <v>156</v>
       </c>
-      <c r="H3" s="16" t="s">
-        <v>85</v>
-      </c>
-      <c r="I3" s="16" t="s">
+      <c r="J3" s="24" t="s">
         <v>157</v>
       </c>
-      <c r="J3" s="16" t="s">
+      <c r="K3" s="24" t="s">
         <v>158</v>
       </c>
-      <c r="K3" s="16" t="s">
+      <c r="L3" s="24" t="s">
+        <v>10</v>
+      </c>
+      <c r="M3" s="24" t="s">
         <v>159</v>
       </c>
-      <c r="L3" s="16" t="s">
+      <c r="N3" s="24" t="s">
         <v>11</v>
       </c>
-      <c r="M3" s="16" t="s">
-        <v>160</v>
-      </c>
-      <c r="N3" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="O3" s="16" t="s">
-        <v>22</v>
-      </c>
-      <c r="P3" s="1" t="s">
+      <c r="O3" s="29" t="s">
+        <v>21</v>
+      </c>
+      <c r="P3" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q3" s="29" t="s">
         <v>20</v>
       </c>
-      <c r="Q3" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="R3" s="16" t="s">
-        <v>24</v>
+      <c r="R3" s="29" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="4" spans="1:18" ht="15.75" x14ac:dyDescent="0.3">
@@ -2290,23 +2400,23 @@
         <v>0</v>
       </c>
       <c r="B4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D4" t="str">
         <f t="shared" ref="D4:D12" si="0">_xlfn.CONCAT(B4,":",C4)</f>
         <v>Industrial_roundwood:FI</v>
       </c>
       <c r="E4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F4">
         <v>0</v>
       </c>
       <c r="H4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="M4" s="4"/>
       <c r="P4">
@@ -2316,7 +2426,7 @@
         <v>0.34699999999999998</v>
       </c>
       <c r="R4" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="5" spans="1:18" ht="15.75" x14ac:dyDescent="0.3">
@@ -2324,23 +2434,23 @@
         <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D5" t="str">
         <f t="shared" si="0"/>
         <v>Sawmilling:FI</v>
       </c>
       <c r="E5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F5">
         <v>0</v>
       </c>
       <c r="H5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="M5" s="4"/>
       <c r="P5">
@@ -2350,7 +2460,7 @@
         <v>0.39200000000000002</v>
       </c>
       <c r="R5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.25">
@@ -2358,23 +2468,23 @@
         <v>2</v>
       </c>
       <c r="B6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D6" t="str">
         <f t="shared" si="0"/>
         <v>Residues:FI</v>
       </c>
       <c r="E6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F6">
         <v>0</v>
       </c>
       <c r="H6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="P6">
         <v>0.40899999999999997</v>
@@ -2383,7 +2493,7 @@
         <v>0.05</v>
       </c>
       <c r="R6" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.25">
@@ -2391,23 +2501,23 @@
         <v>3</v>
       </c>
       <c r="B7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D7" t="str">
         <f t="shared" si="0"/>
         <v>Sawnwood:FI</v>
       </c>
       <c r="E7" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F7">
         <v>0</v>
       </c>
       <c r="H7" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="P7">
         <v>0.40899999999999997</v>
@@ -2416,7 +2526,7 @@
         <v>0.53200000000000003</v>
       </c>
       <c r="R7" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="8" spans="1:18" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -2424,26 +2534,26 @@
         <v>4</v>
       </c>
       <c r="B8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C8" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D8" t="str">
         <f t="shared" si="0"/>
         <v>Construction:FI</v>
       </c>
       <c r="E8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F8">
         <v>10</v>
       </c>
       <c r="H8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I8" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="P8">
         <v>0.752</v>
@@ -2452,7 +2562,7 @@
         <v>0.44400000000000001</v>
       </c>
       <c r="R8" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="9" spans="1:18" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -2460,26 +2570,26 @@
         <v>5</v>
       </c>
       <c r="B9" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D9" t="str">
         <f t="shared" si="0"/>
         <v>Furniture:FI</v>
       </c>
       <c r="E9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F9">
         <v>5</v>
       </c>
       <c r="H9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I9" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="P9">
         <v>0.65600000000000003</v>
@@ -2488,7 +2598,7 @@
         <v>0.77300000000000002</v>
       </c>
       <c r="R9" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.25">
@@ -2496,23 +2606,23 @@
         <v>6</v>
       </c>
       <c r="B10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D10" t="str">
         <f t="shared" si="0"/>
         <v>Sawnwood:Import</v>
       </c>
       <c r="E10" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F10">
         <v>0</v>
       </c>
       <c r="H10" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="P10">
         <v>0.24299999999999999</v>
@@ -2521,7 +2631,7 @@
         <v>0.9</v>
       </c>
       <c r="R10" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.25">
@@ -2529,23 +2639,23 @@
         <v>7</v>
       </c>
       <c r="B11" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D11" t="str">
         <f t="shared" si="0"/>
         <v>Sawnwood:Export</v>
       </c>
       <c r="E11" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F11">
         <v>0</v>
       </c>
       <c r="H11" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="P11">
         <v>0.69099999999999995</v>
@@ -2554,7 +2664,7 @@
         <v>0.16500000000000001</v>
       </c>
       <c r="R11" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.25">
@@ -2562,23 +2672,23 @@
         <v>8</v>
       </c>
       <c r="B12" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C12" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D12" t="str">
         <f t="shared" si="0"/>
         <v>Incineration:FI</v>
       </c>
       <c r="E12" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F12">
         <v>0</v>
       </c>
       <c r="H12" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="P12">
         <v>0.96599999999999997</v>
@@ -2587,7 +2697,7 @@
         <v>0.48299999999999998</v>
       </c>
       <c r="R12" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="18" ht="15.6" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -2614,7 +2724,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B692AEE8-68EE-4B81-A49D-50BF066DFFE7}">
   <dimension ref="A1:P91"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2638,7 +2748,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="27" t="s">
         <v>4</v>
       </c>
       <c r="B1" s="2" t="s">
@@ -2674,10 +2784,10 @@
       <c r="L1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="M1" s="23" t="s">
         <v>5</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="N1" s="23" t="s">
         <v>5</v>
       </c>
       <c r="O1" s="2" t="s">
@@ -2688,7 +2798,7 @@
       </c>
     </row>
     <row r="2" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="27" t="s">
         <v>8</v>
       </c>
       <c r="B2" s="2"/>
@@ -2701,89 +2811,93 @@
       <c r="I2" s="2"/>
       <c r="J2" s="2"/>
       <c r="K2" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="L2" s="2"/>
-      <c r="M2" s="2"/>
-      <c r="N2" s="2"/>
+      <c r="M2" s="23" t="s">
+        <v>240</v>
+      </c>
+      <c r="N2" s="23" t="s">
+        <v>240</v>
+      </c>
       <c r="O2" s="2" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="P2" s="2"/>
     </row>
     <row r="3" spans="1:16" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="15" t="s">
-        <v>184</v>
+      <c r="A3" s="28" t="s">
+        <v>183</v>
       </c>
       <c r="B3" s="9" t="s">
+        <v>164</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="D3" s="9" t="s">
         <v>165</v>
       </c>
-      <c r="C3" s="9" t="s">
-        <v>155</v>
-      </c>
-      <c r="D3" s="9" t="s">
+      <c r="E3" s="9" t="s">
         <v>166</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="F3" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="G3" s="9" t="s">
         <v>167</v>
       </c>
-      <c r="F3" s="9" t="s">
-        <v>155</v>
-      </c>
-      <c r="G3" s="9" t="s">
+      <c r="H3" s="9" t="s">
         <v>168</v>
       </c>
-      <c r="H3" s="9" t="s">
+      <c r="I3" s="9" t="s">
         <v>169</v>
       </c>
-      <c r="I3" s="9" t="s">
-        <v>170</v>
-      </c>
       <c r="J3" s="9" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="K3" s="9" t="s">
         <v>8</v>
       </c>
       <c r="L3" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="M3" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="M3" s="25" t="s">
+        <v>170</v>
+      </c>
+      <c r="N3" s="26" t="s">
         <v>171</v>
       </c>
-      <c r="N3" s="10" t="s">
-        <v>172</v>
-      </c>
       <c r="O3" s="11" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="P3" s="12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C4" t="str">
         <f>+_xlfn.XLOOKUP(H4,Processes!$D$4:$D$47,Processes!$E$4:$E$47)</f>
         <v>Source</v>
       </c>
       <c r="D4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F4" t="str">
         <f>+_xlfn.XLOOKUP(I4,Processes!$D$4:$D$47,Processes!$E$4:$E$47)</f>
         <v>First</v>
       </c>
       <c r="G4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H4" s="3" t="str">
         <f t="shared" ref="H4:H13" si="0">_xlfn.CONCAT(B4,":",D4)</f>
@@ -2797,39 +2911,39 @@
         <v>60</v>
       </c>
       <c r="K4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L4">
         <v>2021</v>
       </c>
       <c r="N4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="P4" s="13"/>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C5" t="str">
         <f>+_xlfn.XLOOKUP(H5,Processes!$D$4:$D$47,Processes!$E$4:$E$47)</f>
         <v>First</v>
       </c>
       <c r="D5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F5" t="str">
         <f>+_xlfn.XLOOKUP(I5,Processes!$D$4:$D$47,Processes!$E$4:$E$47)</f>
         <v>Second</v>
       </c>
       <c r="G5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H5" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2849,33 +2963,33 @@
         <v>2021</v>
       </c>
       <c r="N5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="P5" s="13"/>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B6" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C6" t="str">
         <f>+_xlfn.XLOOKUP(H6,Processes!$D$4:$D$47,Processes!$E$4:$E$47)</f>
         <v>First</v>
       </c>
       <c r="D6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F6" t="str">
         <f>+_xlfn.XLOOKUP(I6,Processes!$D$4:$D$47,Processes!$E$4:$E$47)</f>
         <v>by_prod</v>
       </c>
       <c r="G6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H6" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2889,39 +3003,39 @@
         <v>10</v>
       </c>
       <c r="K6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L6">
         <v>2021</v>
       </c>
       <c r="N6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="P6" s="13"/>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C7" t="str">
         <f>+_xlfn.XLOOKUP(H7,Processes!$D$4:$D$47,Processes!$E$4:$E$47)</f>
         <v>Second</v>
       </c>
       <c r="D7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F7" t="str">
         <f>+_xlfn.XLOOKUP(I7,Processes!$D$4:$D$47,Processes!$E$4:$E$47)</f>
         <v>VAM</v>
       </c>
       <c r="G7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H7" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2941,7 +3055,7 @@
         <v>2021</v>
       </c>
       <c r="N7" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="O7">
         <v>0.22500000000000001</v>
@@ -2949,27 +3063,27 @@
     </row>
     <row r="8" spans="1:16" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B8" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C8" t="str">
         <f>+_xlfn.XLOOKUP(H8,Processes!$D$4:$D$47,Processes!$E$4:$E$47)</f>
         <v>Second</v>
       </c>
       <c r="D8" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F8" t="str">
         <f>+_xlfn.XLOOKUP(I8,Processes!$D$4:$D$47,Processes!$E$4:$E$47)</f>
         <v>VAM</v>
       </c>
       <c r="G8" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H8" s="3" t="str">
         <f>_xlfn.CONCAT(B8,":",D8)</f>
@@ -2989,7 +3103,7 @@
         <v>2021</v>
       </c>
       <c r="N8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="O8">
         <v>0.22500000000000001</v>
@@ -2997,27 +3111,27 @@
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C9" t="str">
         <f>+_xlfn.XLOOKUP(H9,Processes!$D$4:$D$47,Processes!$E$4:$E$47)</f>
         <v>VAM</v>
       </c>
       <c r="D9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F9" t="str">
         <f>+_xlfn.XLOOKUP(I9,Processes!$D$4:$D$47,Processes!$E$4:$E$47)</f>
         <v>First</v>
       </c>
       <c r="G9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H9" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3037,32 +3151,32 @@
         <v>2021</v>
       </c>
       <c r="N9" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="10" spans="1:16" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C10" t="str">
         <f>+_xlfn.XLOOKUP(H10,Processes!$D$4:$D$47,Processes!$E$4:$E$47)</f>
         <v>VAM</v>
       </c>
       <c r="D10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E10" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F10" t="str">
         <f>+_xlfn.XLOOKUP(I10,Processes!$D$4:$D$47,Processes!$E$4:$E$47)</f>
         <v>EoL</v>
       </c>
       <c r="G10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H10" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3082,31 +3196,31 @@
         <v>2021</v>
       </c>
       <c r="N10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B11" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C11" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D11" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E11" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F11" t="str">
         <f>+_xlfn.XLOOKUP(I11,Processes!$D$4:$D$47,Processes!$E$4:$E$47)</f>
         <v>EoL</v>
       </c>
       <c r="G11" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H11" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3126,33 +3240,33 @@
         <v>2021</v>
       </c>
       <c r="N11" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="P11" s="13"/>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C12" t="str">
         <f>+_xlfn.XLOOKUP(H12,Processes!$D$4:$D$47,Processes!$E$4:$E$47)</f>
         <v>Second</v>
       </c>
       <c r="D12" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F12" t="str">
         <f>+_xlfn.XLOOKUP(I12,Processes!$D$4:$D$47,Processes!$E$4:$E$47)</f>
         <v>RoW</v>
       </c>
       <c r="G12" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H12" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3166,39 +3280,39 @@
         <v>20</v>
       </c>
       <c r="K12" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L12">
         <v>2021</v>
       </c>
       <c r="N12" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="P12" s="13"/>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B13" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C13" t="str">
         <f>+_xlfn.XLOOKUP(H13,Processes!$D$4:$D$47,Processes!$E$4:$E$47)</f>
         <v>RoW</v>
       </c>
       <c r="D13" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E13" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F13" t="str">
         <f>+_xlfn.XLOOKUP(I13,Processes!$D$4:$D$47,Processes!$E$4:$E$47)</f>
         <v>Second</v>
       </c>
       <c r="G13" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H13" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3212,13 +3326,13 @@
         <v>10</v>
       </c>
       <c r="K13" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L13">
         <v>2021</v>
       </c>
       <c r="N13" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="P13" s="13"/>
     </row>
@@ -3613,7 +3727,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD427C93-5971-4A1F-9BA5-0A112F61A8DE}">
   <dimension ref="A1:J4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3629,7 +3743,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="27" t="s">
         <v>4</v>
       </c>
       <c r="B1" s="2" t="s">
@@ -3645,13 +3759,13 @@
         <v>5</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="I1" s="2" t="s">
         <v>5</v>
@@ -3661,7 +3775,7 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="27" t="s">
         <v>8</v>
       </c>
       <c r="B2" s="2"/>
@@ -3675,35 +3789,35 @@
       <c r="J2" s="2"/>
     </row>
     <row r="3" spans="1:10" ht="60.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="15" t="s">
+      <c r="A3" s="28" t="s">
+        <v>215</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="F3" s="9" t="s">
         <v>216</v>
       </c>
-      <c r="B3" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="C3" s="9" t="s">
-        <v>60</v>
-      </c>
-      <c r="D3" s="9" t="s">
-        <v>111</v>
-      </c>
-      <c r="E3" s="9" t="s">
-        <v>112</v>
-      </c>
-      <c r="F3" s="9" t="s">
+      <c r="G3" s="9" t="s">
         <v>217</v>
       </c>
-      <c r="G3" s="9" t="s">
+      <c r="H3" s="9" t="s">
         <v>218</v>
       </c>
-      <c r="H3" s="9" t="s">
+      <c r="I3" s="10" t="s">
         <v>219</v>
       </c>
-      <c r="I3" s="10" t="s">
-        <v>220</v>
-      </c>
       <c r="J3" s="9" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
@@ -3731,7 +3845,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{715F83D3-09E8-436B-8662-E6CF9B40F02C}">
   <dimension ref="A1:D91"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3743,17 +3857,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B1" t="s">
-        <v>42</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="A1" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1" s="9" t="s">
         <v>20</v>
-      </c>
-      <c r="D1" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -3761,7 +3875,7 @@
         <v>2021</v>
       </c>
       <c r="B2" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C2">
         <v>3.6999999999999998E-2</v>
@@ -3775,7 +3889,7 @@
         <v>2021</v>
       </c>
       <c r="B3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C3">
         <v>0.24299999999999999</v>
@@ -3789,7 +3903,7 @@
         <v>2021</v>
       </c>
       <c r="B4" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C4">
         <v>0.40899999999999997</v>
@@ -3803,7 +3917,7 @@
         <v>2021</v>
       </c>
       <c r="B5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C5">
         <v>0.40899999999999997</v>
@@ -3817,7 +3931,7 @@
         <v>2021</v>
       </c>
       <c r="B6" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C6">
         <v>0.752</v>
@@ -3831,7 +3945,7 @@
         <v>2021</v>
       </c>
       <c r="B7" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C7">
         <v>0.65600000000000003</v>
@@ -3845,7 +3959,7 @@
         <v>2021</v>
       </c>
       <c r="B8" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C8">
         <v>0.96599999999999997</v>
@@ -3859,7 +3973,7 @@
         <v>2021</v>
       </c>
       <c r="B9" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C9">
         <v>0.69099999999999995</v>
@@ -3873,7 +3987,7 @@
         <v>2021</v>
       </c>
       <c r="B10" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C10">
         <v>0.24299999999999999</v>
@@ -3887,7 +4001,7 @@
         <v>2022</v>
       </c>
       <c r="B11" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C11">
         <v>3.6999999999999998E-2</v>
@@ -3901,7 +4015,7 @@
         <v>2022</v>
       </c>
       <c r="B12" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C12">
         <v>0.24299999999999999</v>
@@ -3915,7 +4029,7 @@
         <v>2022</v>
       </c>
       <c r="B13" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C13">
         <v>0.40899999999999997</v>
@@ -3929,7 +4043,7 @@
         <v>2022</v>
       </c>
       <c r="B14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C14">
         <v>0.40899999999999997</v>
@@ -3943,7 +4057,7 @@
         <v>2022</v>
       </c>
       <c r="B15" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C15">
         <v>0.752</v>
@@ -3957,7 +4071,7 @@
         <v>2022</v>
       </c>
       <c r="B16" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C16">
         <v>0.65600000000000003</v>
@@ -3971,7 +4085,7 @@
         <v>2022</v>
       </c>
       <c r="B17" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C17">
         <v>0.96599999999999997</v>
@@ -3985,7 +4099,7 @@
         <v>2022</v>
       </c>
       <c r="B18" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C18">
         <v>0.69099999999999995</v>
@@ -3999,7 +4113,7 @@
         <v>2022</v>
       </c>
       <c r="B19" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C19">
         <v>0.24299999999999999</v>
@@ -4013,7 +4127,7 @@
         <v>2023</v>
       </c>
       <c r="B20" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C20">
         <v>3.6999999999999998E-2</v>
@@ -4027,7 +4141,7 @@
         <v>2023</v>
       </c>
       <c r="B21" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C21">
         <v>0.24299999999999999</v>
@@ -4041,7 +4155,7 @@
         <v>2023</v>
       </c>
       <c r="B22" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C22">
         <v>0.40899999999999997</v>
@@ -4055,7 +4169,7 @@
         <v>2023</v>
       </c>
       <c r="B23" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C23">
         <v>0.40899999999999997</v>
@@ -4069,7 +4183,7 @@
         <v>2023</v>
       </c>
       <c r="B24" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C24">
         <v>0.752</v>
@@ -4083,7 +4197,7 @@
         <v>2023</v>
       </c>
       <c r="B25" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C25">
         <v>0.65600000000000003</v>
@@ -4097,7 +4211,7 @@
         <v>2023</v>
       </c>
       <c r="B26" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C26">
         <v>0.96599999999999997</v>
@@ -4111,7 +4225,7 @@
         <v>2023</v>
       </c>
       <c r="B27" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C27">
         <v>0.69099999999999995</v>
@@ -4125,7 +4239,7 @@
         <v>2023</v>
       </c>
       <c r="B28" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C28">
         <v>0.24299999999999999</v>
@@ -4139,7 +4253,7 @@
         <v>2024</v>
       </c>
       <c r="B29" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C29">
         <v>3.6999999999999998E-2</v>
@@ -4153,7 +4267,7 @@
         <v>2024</v>
       </c>
       <c r="B30" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C30">
         <v>0.24299999999999999</v>
@@ -4167,7 +4281,7 @@
         <v>2024</v>
       </c>
       <c r="B31" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C31">
         <v>0.40899999999999997</v>
@@ -4181,7 +4295,7 @@
         <v>2024</v>
       </c>
       <c r="B32" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C32">
         <v>0.40899999999999997</v>
@@ -4195,7 +4309,7 @@
         <v>2024</v>
       </c>
       <c r="B33" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C33">
         <v>0.752</v>
@@ -4209,7 +4323,7 @@
         <v>2024</v>
       </c>
       <c r="B34" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C34">
         <v>0.65600000000000003</v>
@@ -4223,7 +4337,7 @@
         <v>2024</v>
       </c>
       <c r="B35" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C35">
         <v>0.96599999999999997</v>
@@ -4237,7 +4351,7 @@
         <v>2024</v>
       </c>
       <c r="B36" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C36">
         <v>0.69099999999999995</v>
@@ -4251,7 +4365,7 @@
         <v>2024</v>
       </c>
       <c r="B37" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C37">
         <v>0.24299999999999999</v>
@@ -4265,7 +4379,7 @@
         <v>2025</v>
       </c>
       <c r="B38" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C38">
         <v>3.6999999999999998E-2</v>
@@ -4279,7 +4393,7 @@
         <v>2025</v>
       </c>
       <c r="B39" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C39">
         <v>0.24299999999999999</v>
@@ -4293,7 +4407,7 @@
         <v>2025</v>
       </c>
       <c r="B40" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C40">
         <v>0.40899999999999997</v>
@@ -4307,7 +4421,7 @@
         <v>2025</v>
       </c>
       <c r="B41" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C41">
         <v>0.40899999999999997</v>
@@ -4321,7 +4435,7 @@
         <v>2025</v>
       </c>
       <c r="B42" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C42">
         <v>0.752</v>
@@ -4335,7 +4449,7 @@
         <v>2025</v>
       </c>
       <c r="B43" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C43">
         <v>0.65600000000000003</v>
@@ -4349,7 +4463,7 @@
         <v>2025</v>
       </c>
       <c r="B44" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C44">
         <v>0.96599999999999997</v>
@@ -4363,7 +4477,7 @@
         <v>2025</v>
       </c>
       <c r="B45" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C45">
         <v>0.69099999999999995</v>
@@ -4377,7 +4491,7 @@
         <v>2025</v>
       </c>
       <c r="B46" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C46">
         <v>0.24299999999999999</v>
@@ -4391,7 +4505,7 @@
         <v>2026</v>
       </c>
       <c r="B47" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C47">
         <v>3.6999999999999998E-2</v>
@@ -4405,7 +4519,7 @@
         <v>2026</v>
       </c>
       <c r="B48" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C48">
         <v>0.24299999999999999</v>
@@ -4419,7 +4533,7 @@
         <v>2026</v>
       </c>
       <c r="B49" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C49">
         <v>0.40899999999999997</v>
@@ -4433,7 +4547,7 @@
         <v>2026</v>
       </c>
       <c r="B50" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C50">
         <v>0.40899999999999997</v>
@@ -4447,7 +4561,7 @@
         <v>2026</v>
       </c>
       <c r="B51" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C51">
         <v>0.752</v>
@@ -4461,7 +4575,7 @@
         <v>2026</v>
       </c>
       <c r="B52" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C52">
         <v>0.65600000000000003</v>
@@ -4475,7 +4589,7 @@
         <v>2026</v>
       </c>
       <c r="B53" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C53">
         <v>0.96599999999999997</v>
@@ -4489,7 +4603,7 @@
         <v>2026</v>
       </c>
       <c r="B54" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C54">
         <v>0.69099999999999995</v>
@@ -4503,7 +4617,7 @@
         <v>2026</v>
       </c>
       <c r="B55" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C55">
         <v>0.24299999999999999</v>
@@ -4517,7 +4631,7 @@
         <v>2027</v>
       </c>
       <c r="B56" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C56">
         <v>3.6999999999999998E-2</v>
@@ -4531,7 +4645,7 @@
         <v>2027</v>
       </c>
       <c r="B57" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C57">
         <v>0.24299999999999999</v>
@@ -4545,7 +4659,7 @@
         <v>2027</v>
       </c>
       <c r="B58" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C58">
         <v>0.40899999999999997</v>
@@ -4559,7 +4673,7 @@
         <v>2027</v>
       </c>
       <c r="B59" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C59">
         <v>0.40899999999999997</v>
@@ -4573,7 +4687,7 @@
         <v>2027</v>
       </c>
       <c r="B60" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C60">
         <v>0.752</v>
@@ -4587,7 +4701,7 @@
         <v>2027</v>
       </c>
       <c r="B61" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C61">
         <v>0.65600000000000003</v>
@@ -4601,7 +4715,7 @@
         <v>2027</v>
       </c>
       <c r="B62" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C62">
         <v>0.96599999999999997</v>
@@ -4615,7 +4729,7 @@
         <v>2027</v>
       </c>
       <c r="B63" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C63">
         <v>0.69099999999999995</v>
@@ -4629,7 +4743,7 @@
         <v>2027</v>
       </c>
       <c r="B64" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C64">
         <v>0.24299999999999999</v>
@@ -4643,7 +4757,7 @@
         <v>2028</v>
       </c>
       <c r="B65" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C65">
         <v>3.6999999999999998E-2</v>
@@ -4657,7 +4771,7 @@
         <v>2028</v>
       </c>
       <c r="B66" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C66">
         <v>0.24299999999999999</v>
@@ -4671,7 +4785,7 @@
         <v>2028</v>
       </c>
       <c r="B67" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C67">
         <v>0.40899999999999997</v>
@@ -4685,7 +4799,7 @@
         <v>2028</v>
       </c>
       <c r="B68" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C68">
         <v>0.40899999999999997</v>
@@ -4699,7 +4813,7 @@
         <v>2028</v>
       </c>
       <c r="B69" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C69">
         <v>0.752</v>
@@ -4713,7 +4827,7 @@
         <v>2028</v>
       </c>
       <c r="B70" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C70">
         <v>0.65600000000000003</v>
@@ -4727,7 +4841,7 @@
         <v>2028</v>
       </c>
       <c r="B71" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C71">
         <v>0.96599999999999997</v>
@@ -4741,7 +4855,7 @@
         <v>2028</v>
       </c>
       <c r="B72" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C72">
         <v>0.69099999999999995</v>
@@ -4755,7 +4869,7 @@
         <v>2028</v>
       </c>
       <c r="B73" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C73">
         <v>0.24299999999999999</v>
@@ -4769,7 +4883,7 @@
         <v>2029</v>
       </c>
       <c r="B74" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C74">
         <v>3.6999999999999998E-2</v>
@@ -4783,7 +4897,7 @@
         <v>2029</v>
       </c>
       <c r="B75" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C75">
         <v>0.24299999999999999</v>
@@ -4797,7 +4911,7 @@
         <v>2029</v>
       </c>
       <c r="B76" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C76">
         <v>0.40899999999999997</v>
@@ -4811,7 +4925,7 @@
         <v>2029</v>
       </c>
       <c r="B77" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C77">
         <v>0.40899999999999997</v>
@@ -4825,7 +4939,7 @@
         <v>2029</v>
       </c>
       <c r="B78" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C78">
         <v>0.752</v>
@@ -4839,7 +4953,7 @@
         <v>2029</v>
       </c>
       <c r="B79" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C79">
         <v>0.65600000000000003</v>
@@ -4853,7 +4967,7 @@
         <v>2029</v>
       </c>
       <c r="B80" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C80">
         <v>0.96599999999999997</v>
@@ -4867,7 +4981,7 @@
         <v>2029</v>
       </c>
       <c r="B81" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C81">
         <v>0.69099999999999995</v>
@@ -4881,7 +4995,7 @@
         <v>2029</v>
       </c>
       <c r="B82" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C82">
         <v>0.24299999999999999</v>
@@ -4895,7 +5009,7 @@
         <v>2030</v>
       </c>
       <c r="B83" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C83">
         <v>3.6999999999999998E-2</v>
@@ -4909,7 +5023,7 @@
         <v>2030</v>
       </c>
       <c r="B84" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C84">
         <v>0.24299999999999999</v>
@@ -4923,7 +5037,7 @@
         <v>2030</v>
       </c>
       <c r="B85" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C85">
         <v>0.40899999999999997</v>
@@ -4937,7 +5051,7 @@
         <v>2030</v>
       </c>
       <c r="B86" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C86">
         <v>0.40899999999999997</v>
@@ -4951,7 +5065,7 @@
         <v>2030</v>
       </c>
       <c r="B87" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C87">
         <v>0.752</v>
@@ -4965,7 +5079,7 @@
         <v>2030</v>
       </c>
       <c r="B88" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C88">
         <v>0.65600000000000003</v>
@@ -4979,7 +5093,7 @@
         <v>2030</v>
       </c>
       <c r="B89" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C89">
         <v>0.96599999999999997</v>
@@ -4993,7 +5107,7 @@
         <v>2030</v>
       </c>
       <c r="B90" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C90">
         <v>0.69099999999999995</v>
@@ -5007,7 +5121,7 @@
         <v>2030</v>
       </c>
       <c r="B91" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C91">
         <v>0.24299999999999999</v>
@@ -5018,100 +5132,102 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{43406F76-D4E1-4DE8-A811-C2AB881D41ED}">
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="52.85546875" customWidth="1"/>
-    <col min="2" max="2" width="16.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="23.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="37.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="12" width="52.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="41.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="32.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="37.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="13" width="52.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A1" s="25" t="s">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1" s="27"/>
+      <c r="B1" s="30" t="s">
+        <v>105</v>
+      </c>
+      <c r="C1" s="30" t="s">
         <v>106</v>
       </c>
-      <c r="B1" s="25" t="s">
+      <c r="D1" s="30" t="s">
         <v>107</v>
       </c>
-      <c r="C1" s="25" t="s">
+      <c r="E1" s="30" t="s">
         <v>108</v>
       </c>
-      <c r="D1" s="25" t="s">
+      <c r="F1" s="30" t="s">
+        <v>186</v>
+      </c>
+      <c r="G1" s="30" t="s">
         <v>109</v>
       </c>
-      <c r="E1" s="25" t="s">
-        <v>187</v>
-      </c>
-      <c r="F1" s="25" t="s">
+      <c r="H1" s="30" t="s">
         <v>110</v>
       </c>
-      <c r="G1" s="25" t="s">
+      <c r="I1" s="30" t="s">
         <v>111</v>
       </c>
-      <c r="H1" s="25" t="s">
+      <c r="J1" s="30" t="s">
         <v>112</v>
       </c>
-      <c r="I1" s="25" t="s">
+      <c r="K1" s="30" t="s">
+        <v>208</v>
+      </c>
+      <c r="L1" s="30" t="s">
         <v>113</v>
       </c>
-      <c r="J1" s="25" t="s">
-        <v>209</v>
-      </c>
-      <c r="K1" s="25" t="s">
-        <v>114</v>
-      </c>
-      <c r="L1" s="25" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>180</v>
-      </c>
-      <c r="B2" s="3" t="s">
+      <c r="M1" s="30" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+      <c r="A2" s="28" t="s">
+        <v>249</v>
+      </c>
+      <c r="B2" t="s">
+        <v>179</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D2" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="C2" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="D2">
+      <c r="E2">
         <v>-50</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>9</v>
       </c>
-      <c r="G2">
+      <c r="H2">
         <v>2025</v>
       </c>
-      <c r="H2">
+      <c r="I2">
         <v>2030</v>
       </c>
-      <c r="I2" t="s">
-        <v>120</v>
-      </c>
-      <c r="J2" s="24" t="b">
+      <c r="J2" t="s">
+        <v>119</v>
+      </c>
+      <c r="K2" s="22" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-    </row>
   </sheetData>
-  <conditionalFormatting sqref="J2">
+  <conditionalFormatting sqref="K2">
     <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
       <formula>TRUE</formula>
     </cfRule>
@@ -5120,7 +5236,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2" xr:uid="{008CAED9-3C22-4095-9218-2455CD3CED8E}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K2" xr:uid="{008CAED9-3C22-4095-9218-2455CD3CED8E}">
       <formula1>Boolean</formula1>
     </dataValidation>
   </dataValidations>
@@ -5128,17 +5244,17 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{283A9876-07D1-4356-BD7B-618A4AD94BB4}">
+          <x14:formula1>
+            <xm:f>'Data validation parameters'!$F$6:$F$9</xm:f>
+          </x14:formula1>
+          <xm:sqref>I1:J2 I5:J1048576</xm:sqref>
+        </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{21908276-F864-4CA4-BA65-3DBA76B06B97}">
           <x14:formula1>
             <xm:f>'Data validation parameters'!$E$6:$E$7</xm:f>
           </x14:formula1>
-          <xm:sqref>F2:F1048576</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{283A9876-07D1-4356-BD7B-618A4AD94BB4}">
-          <x14:formula1>
-            <xm:f>'Data validation parameters'!$F$6:$F$9</xm:f>
-          </x14:formula1>
-          <xm:sqref>I2:I1048576 J3:J1048576</xm:sqref>
+          <xm:sqref>G2 F1:F2 F5:F1048576</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -5146,7 +5262,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA92C4F1-884F-4740-8793-4A0AB47EED3D}">
   <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -5156,78 +5272,78 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="B1" s="9" t="s">
         <v>136</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B3" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B4" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B5" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B7" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B8" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B9" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C9" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
   </sheetData>
@@ -5236,7 +5352,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C12935D7-39CC-4336-870D-98DAC14A69ED}">
   <dimension ref="B2:H13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -5253,126 +5369,126 @@
   <sheetData>
     <row r="2" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="3" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="5" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B5" s="16" t="s">
+        <v>84</v>
+      </c>
+      <c r="C5" s="16" t="s">
+        <v>72</v>
+      </c>
+      <c r="D5" s="16" t="s">
+        <v>93</v>
+      </c>
+      <c r="E5" s="16" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="5" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B5" s="18" t="s">
-        <v>85</v>
-      </c>
-      <c r="C5" s="18" t="s">
-        <v>73</v>
-      </c>
-      <c r="D5" s="18" t="s">
-        <v>94</v>
-      </c>
-      <c r="E5" s="18" t="s">
-        <v>118</v>
-      </c>
-      <c r="F5" s="18" t="s">
-        <v>113</v>
-      </c>
-      <c r="G5" s="18" t="s">
-        <v>195</v>
-      </c>
-      <c r="H5" s="18" t="s">
-        <v>221</v>
+      <c r="F5" s="16" t="s">
+        <v>112</v>
+      </c>
+      <c r="G5" s="16" t="s">
+        <v>194</v>
+      </c>
+      <c r="H5" s="16" t="s">
+        <v>220</v>
       </c>
     </row>
     <row r="6" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C6" t="b">
         <v>1</v>
       </c>
       <c r="D6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G6" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="H6" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="7" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C7" t="b">
         <v>0</v>
       </c>
       <c r="D7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E7" t="s">
         <v>9</v>
       </c>
       <c r="F7" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G7" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="H7" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D8" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F8" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="H8" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="9" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D9" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F9" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="10" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="11" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="12" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="13" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
   </sheetData>
@@ -5382,15 +5498,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Asiakirja" ma:contentTypeID="0x010100806C55B750152A459818B636E97A41C3" ma:contentTypeVersion="19" ma:contentTypeDescription="Luo uusi asiakirja." ma:contentTypeScope="" ma:versionID="74fd9cb75cef04cf26a1ff9ddef01b4b">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7536dd80-7d39-48e8-9ae3-b4166f580a2d" xmlns:ns3="145cc194-9bea-4db6-b116-a042a4529fcd" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="afbcbfdd38894bc2ff0644b00c8ec680" ns2:_="" ns3:_="">
     <xsd:import namespace="7536dd80-7d39-48e8-9ae3-b4166f580a2d"/>
@@ -5653,7 +5760,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="7536dd80-7d39-48e8-9ae3-b4166f580a2d">
@@ -5665,15 +5772,16 @@
 </p:properties>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8AB3C6F0-DB35-46F0-8FEB-B5E57B48A727}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D60021C7-CA75-4673-96EA-55284BF81134}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5692,7 +5800,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{557FAA9C-B184-448F-B58D-00E4D46BDD72}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
@@ -5707,4 +5815,12 @@
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8AB3C6F0-DB35-46F0-8FEB-B5E57B48A727}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Fixed: - Updated example scenario file - Added version-parameter - Checks version-parameter existence when reading the scenario file and show error message if that is not found
</commit_message>
<xml_diff>
--- a/src/aiphoria/data/example_scenario.xlsx
+++ b/src/aiphoria/data/example_scenario.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\PythonProjects\aiphoria\src\aiphoria\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9EAEAA4-B353-41EC-82AF-073964581B1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BDEF65C-D804-47C9-8390-EADF02E8DA28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1620" yWindow="2175" windowWidth="21600" windowHeight="11295" xr2:uid="{1000A452-A98F-45C1-B843-91F7F67E097C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1000A452-A98F-45C1-B843-91F7F67E097C}"/>
   </bookViews>
   <sheets>
-    <sheet name="INFO" sheetId="16" r:id="rId1"/>
+    <sheet name="QUICK GUIDE" sheetId="16" r:id="rId1"/>
     <sheet name="Settings" sheetId="11" r:id="rId2"/>
     <sheet name="Processes" sheetId="6" r:id="rId3"/>
     <sheet name="Flows" sheetId="1" r:id="rId4"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="541" uniqueCount="252">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="550" uniqueCount="260">
   <si>
     <t>Years</t>
   </si>
@@ -822,18 +822,6 @@
     <t xml:space="preserve"> kg/m3 (Optional)</t>
   </si>
   <si>
-    <t>This is aiphoria settings file</t>
-  </si>
-  <si>
-    <t>Refer to the aiphoria wiki for the detailed explanation of different sheets.</t>
-  </si>
-  <si>
-    <t>Green colored columns are comment / optional fields and could be left blank or removed.</t>
-  </si>
-  <si>
-    <t>Check what columns are defined as comment columns in Settings-sheet</t>
-  </si>
-  <si>
     <t xml:space="preserve"> </t>
   </si>
   <si>
@@ -850,6 +838,132 @@
   </si>
   <si>
     <t>Number of rows to skip when reading data for Scenarios (e.g. 2). NOTE: Header row must be the first row to read!</t>
+  </si>
+  <si>
+    <t>version</t>
+  </si>
+  <si>
+    <t>Number</t>
+  </si>
+  <si>
+    <t>Scenario file format version. Required when using aiphoria &gt;= 1.1.0</t>
+  </si>
+  <si>
+    <t>Quick quide</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The ignored columns can be controlled with parameters </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ignore_columns_processes</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ignore_columns_flows</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> in Settings-sheet</t>
+    </r>
+  </si>
+  <si>
+    <t>https://github.com/EuropeanForestInstitute/aiphoria/wiki</t>
+  </si>
+  <si>
+    <t>Refer to aiphoria wiki for more in-depth explanation:</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Start by looking into the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Settings</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>-sheet</t>
+    </r>
+  </si>
+  <si>
+    <t>Major changes in versions</t>
+  </si>
+  <si>
+    <t>1.1.0</t>
+  </si>
+  <si>
+    <t>Green colored columns are ignored when reading the Process and Flows sheets</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Parameter </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>version</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is now expected to be in Settings-sheet in scenario files</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -859,7 +973,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -920,6 +1034,14 @@
     <font>
       <sz val="11"/>
       <color theme="5" tint="0.79998168889431442"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="20"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1005,7 +1127,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -1055,6 +1177,8 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1517,40 +1641,71 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83DA9B50-109E-4569-8896-9B271C0F5058}">
-  <dimension ref="A2:B7"/>
+  <dimension ref="A2:C12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B2" t="s">
+    <row r="2" spans="1:3" ht="26.25" x14ac:dyDescent="0.4">
+      <c r="A2" s="31"/>
+      <c r="B2" s="32" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B4" s="16" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B5" s="13" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>242</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B4" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B6" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>246</v>
-      </c>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
-        <v>245</v>
+        <v>255</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B9" s="16" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>257</v>
+      </c>
+      <c r="C10" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C11" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="31"/>
+      <c r="B12" s="31"/>
+      <c r="C12" s="31" t="s">
+        <v>259</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B5" r:id="rId1" xr:uid="{56846949-43F1-4B32-BE35-77EABA53CAA2}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89FFA668-DA1A-459B-BD42-D0D7F7709F0D}">
-  <dimension ref="A2:E42"/>
+  <dimension ref="A2:E44"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.7109375" bestFit="1" customWidth="1"/>
@@ -1594,173 +1749,170 @@
     </row>
     <row r="7" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
-        <v>63</v>
-      </c>
-      <c r="C7" s="21" t="s">
-        <v>1</v>
-      </c>
-      <c r="D7" s="21" t="s">
-        <v>91</v>
+        <v>248</v>
+      </c>
+      <c r="C7">
+        <v>2</v>
+      </c>
+      <c r="D7" t="s">
+        <v>249</v>
       </c>
       <c r="E7" t="s">
-        <v>237</v>
+        <v>250</v>
       </c>
     </row>
     <row r="8" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
-        <v>149</v>
-      </c>
-      <c r="C8" t="s">
-        <v>247</v>
-      </c>
-      <c r="D8" t="s">
-        <v>124</v>
+        <v>63</v>
+      </c>
+      <c r="C8" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="D8" s="21" t="s">
+        <v>91</v>
       </c>
       <c r="E8" t="s">
-        <v>151</v>
+        <v>237</v>
       </c>
     </row>
     <row r="9" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
-        <v>64</v>
-      </c>
-      <c r="C9" s="20">
-        <v>2</v>
-      </c>
-      <c r="D9" s="20" t="s">
-        <v>89</v>
+        <v>149</v>
+      </c>
+      <c r="C9" t="s">
+        <v>243</v>
+      </c>
+      <c r="D9" t="s">
+        <v>124</v>
       </c>
       <c r="E9" t="s">
-        <v>67</v>
+        <v>151</v>
       </c>
     </row>
     <row r="10" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
-        <v>65</v>
-      </c>
-      <c r="C10" s="21" t="s">
+        <v>64</v>
+      </c>
+      <c r="C10" s="20">
         <v>2</v>
       </c>
-      <c r="D10" s="21" t="s">
-        <v>90</v>
+      <c r="D10" s="20" t="s">
+        <v>89</v>
       </c>
       <c r="E10" t="s">
-        <v>236</v>
+        <v>67</v>
       </c>
     </row>
     <row r="11" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
-        <v>150</v>
-      </c>
-      <c r="C11" t="s">
-        <v>248</v>
-      </c>
-      <c r="D11" t="s">
-        <v>124</v>
+        <v>65</v>
+      </c>
+      <c r="C11" s="21" t="s">
+        <v>2</v>
+      </c>
+      <c r="D11" s="21" t="s">
+        <v>90</v>
       </c>
       <c r="E11" t="s">
-        <v>152</v>
+        <v>236</v>
       </c>
     </row>
     <row r="12" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
-        <v>66</v>
-      </c>
-      <c r="C12" s="20">
-        <v>2</v>
-      </c>
-      <c r="D12" s="20" t="s">
-        <v>89</v>
+        <v>150</v>
+      </c>
+      <c r="C12" t="s">
+        <v>244</v>
+      </c>
+      <c r="D12" t="s">
+        <v>124</v>
       </c>
       <c r="E12" t="s">
-        <v>67</v>
+        <v>152</v>
       </c>
     </row>
     <row r="13" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C13" s="20">
-        <v>2021</v>
+        <v>2</v>
       </c>
       <c r="D13" s="20" t="s">
         <v>89</v>
       </c>
       <c r="E13" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="14" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C14" s="20">
-        <v>2030</v>
+        <v>2021</v>
       </c>
       <c r="D14" s="20" t="s">
         <v>89</v>
       </c>
       <c r="E14" t="s">
-        <v>78</v>
+        <v>69</v>
       </c>
     </row>
     <row r="15" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
-        <v>71</v>
-      </c>
-      <c r="C15" s="22" t="b">
-        <v>0</v>
-      </c>
-      <c r="D15" t="s">
-        <v>88</v>
+        <v>70</v>
+      </c>
+      <c r="C15" s="20">
+        <v>2030</v>
+      </c>
+      <c r="D15" s="20" t="s">
+        <v>89</v>
       </c>
       <c r="E15" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
     </row>
     <row r="16" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="C16" s="22" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D16" t="s">
         <v>88</v>
       </c>
       <c r="E16" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
+        <v>74</v>
+      </c>
+      <c r="C17" s="22" t="b">
+        <v>1</v>
+      </c>
+      <c r="D17" t="s">
+        <v>88</v>
+      </c>
+      <c r="E17" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B18" t="s">
         <v>82</v>
       </c>
-      <c r="C17" s="14">
+      <c r="C18" s="14">
         <v>0.1</v>
       </c>
-      <c r="D17" s="20" t="s">
+      <c r="D18" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="E17" t="s">
+      <c r="E18" t="s">
         <v>83</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>198</v>
-      </c>
-      <c r="B18" t="s">
-        <v>172</v>
-      </c>
-      <c r="C18" t="s">
-        <v>180</v>
-      </c>
-      <c r="D18" t="s">
-        <v>90</v>
-      </c>
-      <c r="E18" t="s">
-        <v>175</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
@@ -1768,16 +1920,16 @@
         <v>198</v>
       </c>
       <c r="B19" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C19" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="D19" t="s">
         <v>90</v>
       </c>
       <c r="E19" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
@@ -1785,16 +1937,16 @@
         <v>198</v>
       </c>
       <c r="B20" t="s">
-        <v>76</v>
-      </c>
-      <c r="C20" s="18">
-        <v>-3.6666666666666701</v>
-      </c>
-      <c r="D20" s="18" t="s">
-        <v>92</v>
+        <v>173</v>
+      </c>
+      <c r="C20" t="s">
+        <v>176</v>
+      </c>
+      <c r="D20" t="s">
+        <v>90</v>
       </c>
       <c r="E20" t="s">
-        <v>77</v>
+        <v>174</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
@@ -1802,16 +1954,16 @@
         <v>198</v>
       </c>
       <c r="B21" t="s">
-        <v>86</v>
-      </c>
-      <c r="C21" s="22" t="b">
-        <v>1</v>
-      </c>
-      <c r="D21" t="s">
-        <v>88</v>
+        <v>76</v>
+      </c>
+      <c r="C21" s="18">
+        <v>-3.6666666666666701</v>
+      </c>
+      <c r="D21" s="18" t="s">
+        <v>92</v>
       </c>
       <c r="E21" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
@@ -1819,7 +1971,7 @@
         <v>198</v>
       </c>
       <c r="B22" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C22" s="22" t="b">
         <v>1</v>
@@ -1836,16 +1988,16 @@
         <v>198</v>
       </c>
       <c r="B23" t="s">
-        <v>93</v>
-      </c>
-      <c r="C23" t="s">
-        <v>96</v>
+        <v>85</v>
+      </c>
+      <c r="C23" s="22" t="b">
+        <v>1</v>
       </c>
       <c r="D23" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="E23" t="s">
-        <v>114</v>
+        <v>87</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
@@ -1853,16 +2005,16 @@
         <v>198</v>
       </c>
       <c r="B24" t="s">
-        <v>184</v>
-      </c>
-      <c r="C24" s="22" t="b">
-        <v>1</v>
+        <v>93</v>
+      </c>
+      <c r="C24" t="s">
+        <v>96</v>
       </c>
       <c r="D24" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="E24" t="s">
-        <v>185</v>
+        <v>114</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
@@ -1870,16 +2022,16 @@
         <v>198</v>
       </c>
       <c r="B25" t="s">
-        <v>193</v>
-      </c>
-      <c r="C25" t="s">
-        <v>195</v>
+        <v>184</v>
+      </c>
+      <c r="C25" s="22" t="b">
+        <v>1</v>
       </c>
       <c r="D25" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="E25" t="s">
-        <v>197</v>
+        <v>185</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
@@ -1887,16 +2039,16 @@
         <v>198</v>
       </c>
       <c r="B26" t="s">
-        <v>99</v>
+        <v>193</v>
       </c>
       <c r="C26" t="s">
-        <v>100</v>
+        <v>195</v>
       </c>
       <c r="D26" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E26" t="s">
-        <v>235</v>
+        <v>197</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
@@ -1904,16 +2056,16 @@
         <v>198</v>
       </c>
       <c r="B27" t="s">
-        <v>160</v>
+        <v>99</v>
       </c>
       <c r="C27" t="s">
-        <v>181</v>
+        <v>100</v>
       </c>
       <c r="D27" t="s">
-        <v>124</v>
+        <v>90</v>
       </c>
       <c r="E27" t="s">
-        <v>162</v>
+        <v>235</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
@@ -1921,13 +2073,16 @@
         <v>198</v>
       </c>
       <c r="B28" t="s">
-        <v>250</v>
+        <v>160</v>
+      </c>
+      <c r="C28" t="s">
+        <v>181</v>
       </c>
       <c r="D28" t="s">
-        <v>89</v>
+        <v>124</v>
       </c>
       <c r="E28" t="s">
-        <v>251</v>
+        <v>162</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
@@ -1935,16 +2090,13 @@
         <v>198</v>
       </c>
       <c r="B29" t="s">
-        <v>101</v>
-      </c>
-      <c r="C29" s="22" t="b">
-        <v>1</v>
+        <v>246</v>
       </c>
       <c r="D29" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E29" t="s">
-        <v>102</v>
+        <v>247</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
@@ -1952,7 +2104,7 @@
         <v>198</v>
       </c>
       <c r="B30" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C30" s="22" t="b">
         <v>1</v>
@@ -1961,7 +2113,7 @@
         <v>88</v>
       </c>
       <c r="E30" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
@@ -1969,16 +2121,16 @@
         <v>198</v>
       </c>
       <c r="B31" t="s">
-        <v>122</v>
-      </c>
-      <c r="C31" t="s">
-        <v>125</v>
+        <v>103</v>
+      </c>
+      <c r="C31" s="22" t="b">
+        <v>1</v>
       </c>
       <c r="D31" t="s">
-        <v>124</v>
+        <v>88</v>
       </c>
       <c r="E31" t="s">
-        <v>123</v>
+        <v>104</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
@@ -1986,16 +2138,16 @@
         <v>198</v>
       </c>
       <c r="B32" t="s">
-        <v>142</v>
-      </c>
-      <c r="C32" s="20" t="s">
-        <v>143</v>
-      </c>
-      <c r="D32" s="20" t="s">
-        <v>90</v>
+        <v>122</v>
+      </c>
+      <c r="C32" t="s">
+        <v>125</v>
+      </c>
+      <c r="D32" t="s">
+        <v>124</v>
       </c>
       <c r="E32" t="s">
-        <v>234</v>
+        <v>123</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
@@ -2003,41 +2155,44 @@
         <v>198</v>
       </c>
       <c r="B33" t="s">
-        <v>161</v>
-      </c>
-      <c r="D33" t="s">
-        <v>124</v>
+        <v>142</v>
+      </c>
+      <c r="C33" s="20" t="s">
+        <v>143</v>
+      </c>
+      <c r="D33" s="20" t="s">
+        <v>90</v>
       </c>
       <c r="E33" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>198</v>
       </c>
       <c r="B34" t="s">
-        <v>187</v>
+        <v>161</v>
       </c>
       <c r="D34" t="s">
         <v>124</v>
       </c>
       <c r="E34" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>198</v>
       </c>
       <c r="B35" t="s">
-        <v>238</v>
+        <v>187</v>
       </c>
       <c r="D35" t="s">
         <v>124</v>
       </c>
       <c r="E35" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
@@ -2045,16 +2200,13 @@
         <v>198</v>
       </c>
       <c r="B36" t="s">
-        <v>199</v>
-      </c>
-      <c r="C36" t="s">
-        <v>200</v>
+        <v>238</v>
       </c>
       <c r="D36" t="s">
-        <v>90</v>
+        <v>124</v>
       </c>
       <c r="E36" t="s">
-        <v>233</v>
+        <v>189</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
@@ -2062,16 +2214,16 @@
         <v>198</v>
       </c>
       <c r="B37" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
       <c r="C37" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="D37" t="s">
         <v>90</v>
       </c>
       <c r="E37" t="s">
-        <v>211</v>
+        <v>233</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
@@ -2079,16 +2231,16 @@
         <v>198</v>
       </c>
       <c r="B38" t="s">
-        <v>212</v>
-      </c>
-      <c r="C38" s="22" t="b">
-        <v>1</v>
+        <v>209</v>
+      </c>
+      <c r="C38" t="s">
+        <v>210</v>
       </c>
       <c r="D38" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="E38" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
@@ -2096,7 +2248,7 @@
         <v>198</v>
       </c>
       <c r="B39" t="s">
-        <v>224</v>
+        <v>212</v>
       </c>
       <c r="C39" s="22" t="b">
         <v>1</v>
@@ -2105,7 +2257,7 @@
         <v>88</v>
       </c>
       <c r="E39" t="s">
-        <v>225</v>
+        <v>213</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
@@ -2113,16 +2265,16 @@
         <v>198</v>
       </c>
       <c r="B40" t="s">
-        <v>226</v>
-      </c>
-      <c r="C40" t="s">
-        <v>227</v>
+        <v>224</v>
+      </c>
+      <c r="C40" s="22" t="b">
+        <v>1</v>
       </c>
       <c r="D40" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="E40" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
@@ -2130,16 +2282,16 @@
         <v>198</v>
       </c>
       <c r="B41" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C41" t="s">
-        <v>181</v>
+        <v>227</v>
       </c>
       <c r="D41" t="s">
-        <v>124</v>
+        <v>90</v>
       </c>
       <c r="E41" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
@@ -2147,21 +2299,46 @@
         <v>198</v>
       </c>
       <c r="B42" t="s">
+        <v>228</v>
+      </c>
+      <c r="C42" t="s">
+        <v>181</v>
+      </c>
+      <c r="D42" t="s">
+        <v>124</v>
+      </c>
+      <c r="E42" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>198</v>
+      </c>
+      <c r="B43" t="s">
         <v>230</v>
       </c>
-      <c r="C42">
+      <c r="C43">
         <v>2</v>
       </c>
-      <c r="D42" t="s">
+      <c r="D43" t="s">
         <v>89</v>
       </c>
-      <c r="E42" t="s">
+      <c r="E43" t="s">
         <v>231</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B44" t="s">
+        <v>248</v>
+      </c>
+      <c r="C44">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="B6:E6" xr:uid="{89FFA668-DA1A-459B-BD42-D0D7F7709F0D}"/>
-  <conditionalFormatting sqref="C15:C16">
+  <conditionalFormatting sqref="C16:C17">
     <cfRule type="cellIs" dxfId="11" priority="11" operator="equal">
       <formula>TRUE</formula>
     </cfRule>
@@ -2169,7 +2346,7 @@
       <formula>TRUE</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C21:C22">
+  <conditionalFormatting sqref="C22:C23">
     <cfRule type="cellIs" dxfId="9" priority="9" operator="equal">
       <formula>TRUE</formula>
     </cfRule>
@@ -2177,7 +2354,7 @@
       <formula>TRUE</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C24">
+  <conditionalFormatting sqref="C25">
     <cfRule type="cellIs" dxfId="7" priority="5" operator="equal">
       <formula>TRUE</formula>
     </cfRule>
@@ -2185,7 +2362,7 @@
       <formula>TRUE</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C29:C30">
+  <conditionalFormatting sqref="C30:C31">
     <cfRule type="cellIs" dxfId="5" priority="7" operator="equal">
       <formula>TRUE</formula>
     </cfRule>
@@ -2193,7 +2370,7 @@
       <formula>TRUE</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C38:C39">
+  <conditionalFormatting sqref="C39:C40">
     <cfRule type="cellIs" dxfId="3" priority="3" operator="equal">
       <formula>TRUE</formula>
     </cfRule>
@@ -2202,12 +2379,12 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C15:C16 C21:C22 C29:C30 C24 C38:C39" xr:uid="{79A7E31C-3284-4405-9B5F-03E099B07563}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C16:C17 C22:C23 C30:C31 C25 C39:C40" xr:uid="{79A7E31C-3284-4405-9B5F-03E099B07563}">
       <formula1>Boolean</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
@@ -2215,13 +2392,13 @@
           <x14:formula1>
             <xm:f>'Data validation parameters'!$D$6:$D$9</xm:f>
           </x14:formula1>
-          <xm:sqref>C23</xm:sqref>
+          <xm:sqref>C24</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{7A04E2A2-4928-4E28-9F6D-7D556381B8E8}">
           <x14:formula1>
             <xm:f>'Data validation parameters'!$G$6:$G$7</xm:f>
           </x14:formula1>
-          <xm:sqref>C25</xm:sqref>
+          <xm:sqref>C26</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -5196,7 +5373,7 @@
     </row>
     <row r="2" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="28" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
       <c r="B2" t="s">
         <v>179</v>
@@ -5498,6 +5675,27 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7536dd80-7d39-48e8-9ae3-b4166f580a2d">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="145cc194-9bea-4db6-b116-a042a4529fcd" xsi:nil="true"/>
+    <Comment xmlns="7536dd80-7d39-48e8-9ae3-b4166f580a2d" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Asiakirja" ma:contentTypeID="0x010100806C55B750152A459818B636E97A41C3" ma:contentTypeVersion="19" ma:contentTypeDescription="Luo uusi asiakirja." ma:contentTypeScope="" ma:versionID="74fd9cb75cef04cf26a1ff9ddef01b4b">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7536dd80-7d39-48e8-9ae3-b4166f580a2d" xmlns:ns3="145cc194-9bea-4db6-b116-a042a4529fcd" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="afbcbfdd38894bc2ff0644b00c8ec680" ns2:_="" ns3:_="">
     <xsd:import namespace="7536dd80-7d39-48e8-9ae3-b4166f580a2d"/>
@@ -5760,42 +5958,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7536dd80-7d39-48e8-9ae3-b4166f580a2d">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="145cc194-9bea-4db6-b116-a042a4529fcd" xsi:nil="true"/>
-    <Comment xmlns="7536dd80-7d39-48e8-9ae3-b4166f580a2d" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D60021C7-CA75-4673-96EA-55284BF81134}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8AB3C6F0-DB35-46F0-8FEB-B5E57B48A727}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="7536dd80-7d39-48e8-9ae3-b4166f580a2d"/>
-    <ds:schemaRef ds:uri="145cc194-9bea-4db6-b116-a042a4529fcd"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -5818,9 +5984,20 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8AB3C6F0-DB35-46F0-8FEB-B5E57B48A727}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D60021C7-CA75-4673-96EA-55284BF81134}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="7536dd80-7d39-48e8-9ae3-b4166f580a2d"/>
+    <ds:schemaRef ds:uri="145cc194-9bea-4db6-b116-a042a4529fcd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
- Reduced complexity of Flow-object - Updated tests - Updated example scenario - Updated .gitignore
</commit_message>
<xml_diff>
--- a/src/aiphoria/data/example_scenario.xlsx
+++ b/src/aiphoria/data/example_scenario.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\PythonProjects\aiphoria\src\aiphoria\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BDEF65C-D804-47C9-8390-EADF02E8DA28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CAE2671-3DEF-4367-8CB4-0AEF702A6E53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1000A452-A98F-45C1-B843-91F7F67E097C}"/>
   </bookViews>
@@ -24,8 +24,8 @@
     <sheet name="Data validation parameters" sheetId="9" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Flows!$A$3:$P$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Processes!$D$3:$R$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Flows!$A$3:$H$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Processes!$D$3:$L$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Settings!$B$6:$E$6</definedName>
     <definedName name="Boolean">'Data validation parameters'!$C$6:$C$7</definedName>
   </definedNames>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="550" uniqueCount="260">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="484" uniqueCount="240">
   <si>
     <t>Years</t>
   </si>
@@ -82,12 +82,6 @@
     <t>%</t>
   </si>
   <si>
-    <t>Density</t>
-  </si>
-  <si>
-    <t>Modelling status</t>
-  </si>
-  <si>
     <t>Comment</t>
   </si>
   <si>
@@ -164,9 +158,6 @@
   </si>
   <si>
     <t>Normal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Random input values </t>
   </si>
   <si>
     <t>Sawmilling:FI</t>
@@ -561,21 +552,9 @@
     <t>Transformation stage</t>
   </si>
   <si>
-    <t>Lifetime source</t>
-  </si>
-  <si>
     <t>Distribution parameters</t>
   </si>
   <si>
-    <t>Wood content</t>
-  </si>
-  <si>
-    <t>Wood content source</t>
-  </si>
-  <si>
-    <t>Density source</t>
-  </si>
-  <si>
     <t>ignore_columns_scenarios</t>
   </si>
   <si>
@@ -588,30 +567,6 @@
     <t>Ignore Excel columns defined in the list when reading data from Colors sheet. Each column name must be separated by comma (',')</t>
   </si>
   <si>
-    <t>Source process</t>
-  </si>
-  <si>
-    <t>Source process location</t>
-  </si>
-  <si>
-    <t>Target process</t>
-  </si>
-  <si>
-    <t>Target process location</t>
-  </si>
-  <si>
-    <t>Source ID</t>
-  </si>
-  <si>
-    <t>Target ID</t>
-  </si>
-  <si>
-    <t>Data source</t>
-  </si>
-  <si>
-    <t>Data source comment</t>
-  </si>
-  <si>
     <t>baseline_value_name</t>
   </si>
   <si>
@@ -813,22 +768,7 @@
     <t>prioritize_transformation_stages</t>
   </si>
   <si>
-    <t>% (Optional)</t>
-  </si>
-  <si>
-    <t>(Optional)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> kg/m3 (Optional)</t>
-  </si>
-  <si>
     <t xml:space="preserve"> </t>
-  </si>
-  <si>
-    <t>A,G,J,K,L,M,N</t>
-  </si>
-  <si>
-    <t>A,M,N</t>
   </si>
   <si>
     <t>This column is ignored (check parameter ignore_columns_scenarios in Settings-sheet)</t>
@@ -973,7 +913,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1002,12 +942,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF4C4845"/>
-      <name val="Open Sans"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="8"/>
@@ -1125,50 +1059,34 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1177,8 +1095,7 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1299,16 +1216,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>539805</xdr:colOff>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>15</xdr:row>
-      <xdr:rowOff>64113</xdr:rowOff>
+      <xdr:rowOff>6963</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>192604</xdr:colOff>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>1948324</xdr:colOff>
       <xdr:row>31</xdr:row>
-      <xdr:rowOff>167367</xdr:rowOff>
+      <xdr:rowOff>110217</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1331,7 +1248,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2701980" y="2969238"/>
+          <a:off x="3283005" y="3474063"/>
           <a:ext cx="8501524" cy="3151254"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1641,58 +1558,55 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83DA9B50-109E-4569-8896-9B271C0F5058}">
-  <dimension ref="A2:C12"/>
+  <dimension ref="A2:C13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="2" spans="1:3" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="A2" s="31"/>
-      <c r="B2" s="32" t="s">
-        <v>251</v>
+      <c r="B2" s="23" t="s">
+        <v>231</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B4" s="16" t="s">
-        <v>254</v>
+      <c r="B4" s="12" t="s">
+        <v>234</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B5" s="13" t="s">
-        <v>253</v>
+      <c r="B5" s="9" t="s">
+        <v>233</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>242</v>
+        <v>224</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
-        <v>255</v>
+        <v>235</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B9" s="16" t="s">
-        <v>256</v>
+      <c r="B9" s="12" t="s">
+        <v>236</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
-        <v>257</v>
+        <v>237</v>
       </c>
       <c r="C10" t="s">
-        <v>258</v>
+        <v>238</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C11" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="31"/>
-      <c r="B12" s="31"/>
-      <c r="C12" s="31" t="s">
-        <v>259</v>
+        <v>232</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C13" t="s">
+        <v>239</v>
       </c>
     </row>
   </sheetData>
@@ -1716,621 +1630,621 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:5" ht="21" x14ac:dyDescent="0.35">
-      <c r="B2" s="17" t="s">
-        <v>61</v>
+      <c r="B2" s="13" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="3" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B3" s="19" t="s">
-        <v>80</v>
+      <c r="B3" s="15" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="4" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
-        <v>79</v>
-      </c>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
+        <v>76</v>
+      </c>
+      <c r="C4" s="15"/>
+      <c r="D4" s="15"/>
+      <c r="E4" s="15"/>
     </row>
     <row r="6" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B6" s="9" t="s">
-        <v>62</v>
-      </c>
-      <c r="C6" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="D6" s="9" t="s">
-        <v>81</v>
-      </c>
-      <c r="E6" s="9" t="s">
+      <c r="B6" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="E6" s="5" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="7" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
-        <v>248</v>
+        <v>228</v>
       </c>
       <c r="C7">
         <v>2</v>
       </c>
       <c r="D7" t="s">
-        <v>249</v>
+        <v>229</v>
       </c>
       <c r="E7" t="s">
-        <v>250</v>
+        <v>230</v>
       </c>
     </row>
     <row r="8" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
-        <v>63</v>
-      </c>
-      <c r="C8" s="21" t="s">
+        <v>60</v>
+      </c>
+      <c r="C8" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="D8" s="21" t="s">
-        <v>91</v>
+      <c r="D8" s="17" t="s">
+        <v>88</v>
       </c>
       <c r="E8" t="s">
-        <v>237</v>
+        <v>222</v>
       </c>
     </row>
     <row r="9" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="C9" t="s">
-        <v>243</v>
+        <v>166</v>
       </c>
       <c r="D9" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="E9" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
     </row>
     <row r="10" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
+        <v>61</v>
+      </c>
+      <c r="C10" s="16">
+        <v>2</v>
+      </c>
+      <c r="D10" s="16" t="s">
+        <v>86</v>
+      </c>
+      <c r="E10" t="s">
         <v>64</v>
-      </c>
-      <c r="C10" s="20">
-        <v>2</v>
-      </c>
-      <c r="D10" s="20" t="s">
-        <v>89</v>
-      </c>
-      <c r="E10" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="11" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
-        <v>65</v>
-      </c>
-      <c r="C11" s="21" t="s">
+        <v>62</v>
+      </c>
+      <c r="C11" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="D11" s="21" t="s">
-        <v>90</v>
+      <c r="D11" s="17" t="s">
+        <v>87</v>
       </c>
       <c r="E11" t="s">
-        <v>236</v>
+        <v>221</v>
       </c>
     </row>
     <row r="12" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="C12" t="s">
-        <v>244</v>
+        <v>166</v>
       </c>
       <c r="D12" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="E12" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
     </row>
     <row r="13" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
-        <v>66</v>
-      </c>
-      <c r="C13" s="20">
+        <v>63</v>
+      </c>
+      <c r="C13" s="16">
         <v>2</v>
       </c>
-      <c r="D13" s="20" t="s">
-        <v>89</v>
+      <c r="D13" s="16" t="s">
+        <v>86</v>
       </c>
       <c r="E13" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="14" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
-        <v>68</v>
-      </c>
-      <c r="C14" s="20">
+        <v>65</v>
+      </c>
+      <c r="C14" s="16">
         <v>2021</v>
       </c>
-      <c r="D14" s="20" t="s">
-        <v>89</v>
+      <c r="D14" s="16" t="s">
+        <v>86</v>
       </c>
       <c r="E14" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="15" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
-        <v>70</v>
-      </c>
-      <c r="C15" s="20">
+        <v>67</v>
+      </c>
+      <c r="C15" s="16">
         <v>2030</v>
       </c>
-      <c r="D15" s="20" t="s">
-        <v>89</v>
+      <c r="D15" s="16" t="s">
+        <v>86</v>
       </c>
       <c r="E15" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
     </row>
     <row r="16" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
-        <v>71</v>
-      </c>
-      <c r="C16" s="22" t="b">
+        <v>68</v>
+      </c>
+      <c r="C16" s="18" t="b">
         <v>0</v>
       </c>
       <c r="D16" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="E16" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
-        <v>74</v>
-      </c>
-      <c r="C17" s="22" t="b">
+        <v>71</v>
+      </c>
+      <c r="C17" s="18" t="b">
         <v>1</v>
       </c>
       <c r="D17" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="E17" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
-        <v>82</v>
-      </c>
-      <c r="C18" s="14">
+        <v>79</v>
+      </c>
+      <c r="C18" s="10">
         <v>0.1</v>
       </c>
-      <c r="D18" s="20" t="s">
-        <v>92</v>
+      <c r="D18" s="16" t="s">
+        <v>89</v>
       </c>
       <c r="E18" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>198</v>
+        <v>183</v>
       </c>
       <c r="B19" t="s">
-        <v>172</v>
+        <v>157</v>
       </c>
       <c r="C19" t="s">
-        <v>180</v>
+        <v>165</v>
       </c>
       <c r="D19" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="E19" t="s">
-        <v>175</v>
+        <v>160</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>198</v>
+        <v>183</v>
       </c>
       <c r="B20" t="s">
-        <v>173</v>
+        <v>158</v>
       </c>
       <c r="C20" t="s">
-        <v>176</v>
+        <v>161</v>
       </c>
       <c r="D20" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="E20" t="s">
-        <v>174</v>
+        <v>159</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>198</v>
+        <v>183</v>
       </c>
       <c r="B21" t="s">
-        <v>76</v>
-      </c>
-      <c r="C21" s="18">
+        <v>73</v>
+      </c>
+      <c r="C21" s="14">
         <v>-3.6666666666666701</v>
       </c>
-      <c r="D21" s="18" t="s">
-        <v>92</v>
+      <c r="D21" s="14" t="s">
+        <v>89</v>
       </c>
       <c r="E21" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>198</v>
+        <v>183</v>
       </c>
       <c r="B22" t="s">
-        <v>86</v>
-      </c>
-      <c r="C22" s="22" t="b">
+        <v>83</v>
+      </c>
+      <c r="C22" s="18" t="b">
         <v>1</v>
       </c>
       <c r="D22" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="E22" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>198</v>
+        <v>183</v>
       </c>
       <c r="B23" t="s">
+        <v>82</v>
+      </c>
+      <c r="C23" s="18" t="b">
+        <v>1</v>
+      </c>
+      <c r="D23" t="s">
         <v>85</v>
       </c>
-      <c r="C23" s="22" t="b">
-        <v>1</v>
-      </c>
-      <c r="D23" t="s">
-        <v>88</v>
-      </c>
       <c r="E23" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>198</v>
+        <v>183</v>
       </c>
       <c r="B24" t="s">
+        <v>90</v>
+      </c>
+      <c r="C24" t="s">
         <v>93</v>
       </c>
-      <c r="C24" t="s">
-        <v>96</v>
-      </c>
       <c r="D24" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="E24" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>198</v>
+        <v>183</v>
       </c>
       <c r="B25" t="s">
-        <v>184</v>
-      </c>
-      <c r="C25" s="22" t="b">
+        <v>169</v>
+      </c>
+      <c r="C25" s="18" t="b">
         <v>1</v>
       </c>
       <c r="D25" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="E25" t="s">
-        <v>185</v>
+        <v>170</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>198</v>
+        <v>183</v>
       </c>
       <c r="B26" t="s">
-        <v>193</v>
+        <v>178</v>
       </c>
       <c r="C26" t="s">
-        <v>195</v>
+        <v>180</v>
       </c>
       <c r="D26" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="E26" t="s">
-        <v>197</v>
+        <v>182</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>198</v>
+        <v>183</v>
       </c>
       <c r="B27" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="C27" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="D27" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="E27" t="s">
-        <v>235</v>
+        <v>220</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>198</v>
+        <v>183</v>
       </c>
       <c r="B28" t="s">
-        <v>160</v>
+        <v>153</v>
       </c>
       <c r="C28" t="s">
-        <v>181</v>
+        <v>166</v>
       </c>
       <c r="D28" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="E28" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>198</v>
+        <v>183</v>
       </c>
       <c r="B29" t="s">
-        <v>246</v>
+        <v>226</v>
       </c>
       <c r="D29" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="E29" t="s">
-        <v>247</v>
+        <v>227</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>198</v>
+        <v>183</v>
       </c>
       <c r="B30" t="s">
-        <v>101</v>
-      </c>
-      <c r="C30" s="22" t="b">
+        <v>98</v>
+      </c>
+      <c r="C30" s="18" t="b">
         <v>1</v>
       </c>
       <c r="D30" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="E30" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>198</v>
+        <v>183</v>
       </c>
       <c r="B31" t="s">
-        <v>103</v>
-      </c>
-      <c r="C31" s="22" t="b">
+        <v>100</v>
+      </c>
+      <c r="C31" s="18" t="b">
         <v>1</v>
       </c>
       <c r="D31" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="E31" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>198</v>
+        <v>183</v>
       </c>
       <c r="B32" t="s">
+        <v>119</v>
+      </c>
+      <c r="C32" t="s">
         <v>122</v>
       </c>
-      <c r="C32" t="s">
-        <v>125</v>
-      </c>
       <c r="D32" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="E32" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>198</v>
+        <v>183</v>
       </c>
       <c r="B33" t="s">
-        <v>142</v>
-      </c>
-      <c r="C33" s="20" t="s">
-        <v>143</v>
-      </c>
-      <c r="D33" s="20" t="s">
-        <v>90</v>
+        <v>139</v>
+      </c>
+      <c r="C33" s="16" t="s">
+        <v>140</v>
+      </c>
+      <c r="D33" s="16" t="s">
+        <v>87</v>
       </c>
       <c r="E33" t="s">
-        <v>234</v>
+        <v>219</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>198</v>
+        <v>183</v>
       </c>
       <c r="B34" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="D34" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="E34" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>198</v>
+        <v>183</v>
       </c>
       <c r="B35" t="s">
-        <v>187</v>
+        <v>172</v>
       </c>
       <c r="D35" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="E35" t="s">
-        <v>190</v>
+        <v>175</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>198</v>
+        <v>183</v>
       </c>
       <c r="B36" t="s">
-        <v>238</v>
+        <v>223</v>
       </c>
       <c r="D36" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="E36" t="s">
-        <v>189</v>
+        <v>174</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>198</v>
+        <v>183</v>
       </c>
       <c r="B37" t="s">
-        <v>199</v>
+        <v>184</v>
       </c>
       <c r="C37" t="s">
-        <v>200</v>
+        <v>185</v>
       </c>
       <c r="D37" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="E37" t="s">
-        <v>233</v>
+        <v>218</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>198</v>
+        <v>183</v>
       </c>
       <c r="B38" t="s">
-        <v>209</v>
+        <v>194</v>
       </c>
       <c r="C38" t="s">
-        <v>210</v>
+        <v>195</v>
       </c>
       <c r="D38" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="E38" t="s">
-        <v>211</v>
+        <v>196</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
+        <v>183</v>
+      </c>
+      <c r="B39" t="s">
+        <v>197</v>
+      </c>
+      <c r="C39" s="18" t="b">
+        <v>1</v>
+      </c>
+      <c r="D39" t="s">
+        <v>85</v>
+      </c>
+      <c r="E39" t="s">
         <v>198</v>
-      </c>
-      <c r="B39" t="s">
-        <v>212</v>
-      </c>
-      <c r="C39" s="22" t="b">
-        <v>1</v>
-      </c>
-      <c r="D39" t="s">
-        <v>88</v>
-      </c>
-      <c r="E39" t="s">
-        <v>213</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>198</v>
+        <v>183</v>
       </c>
       <c r="B40" t="s">
-        <v>224</v>
-      </c>
-      <c r="C40" s="22" t="b">
+        <v>209</v>
+      </c>
+      <c r="C40" s="18" t="b">
         <v>1</v>
       </c>
       <c r="D40" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="E40" t="s">
-        <v>225</v>
+        <v>210</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>198</v>
+        <v>183</v>
       </c>
       <c r="B41" t="s">
-        <v>226</v>
+        <v>211</v>
       </c>
       <c r="C41" t="s">
-        <v>227</v>
+        <v>212</v>
       </c>
       <c r="D41" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="E41" t="s">
-        <v>232</v>
+        <v>217</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>198</v>
+        <v>183</v>
       </c>
       <c r="B42" t="s">
-        <v>228</v>
+        <v>213</v>
       </c>
       <c r="C42" t="s">
-        <v>181</v>
+        <v>166</v>
       </c>
       <c r="D42" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="E42" t="s">
-        <v>229</v>
+        <v>214</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>198</v>
+        <v>183</v>
       </c>
       <c r="B43" t="s">
-        <v>230</v>
+        <v>215</v>
       </c>
       <c r="C43">
         <v>2</v>
       </c>
       <c r="D43" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="E43" t="s">
-        <v>231</v>
+        <v>216</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B44" t="s">
-        <v>248</v>
+        <v>228</v>
       </c>
       <c r="C44">
         <v>2</v>
@@ -2408,7 +2322,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32C0D592-75C1-4AD1-84F0-2AAE25CA0097}">
-  <dimension ref="A1:R18"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.42578125" bestFit="1" customWidth="1"/>
@@ -2417,21 +2331,15 @@
     <col min="4" max="4" width="23.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="14.7109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="22.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="20.28515625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="16" max="17" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="22.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="19.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A1" s="27"/>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1" s="19"/>
       <c r="B1" s="2" t="s">
         <v>5</v>
       </c>
@@ -2447,43 +2355,27 @@
       <c r="F1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="23"/>
+      <c r="G1" s="2" t="s">
+        <v>5</v>
+      </c>
       <c r="H1" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="I1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="J1" s="23" t="s">
+      <c r="J1" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="K1" s="23" t="s">
+      <c r="L1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="23" t="s">
-        <v>7</v>
-      </c>
-      <c r="M1" s="23" t="s">
-        <v>5</v>
-      </c>
-      <c r="N1" s="23" t="s">
-        <v>5</v>
-      </c>
-      <c r="O1" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="P1" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="Q1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="R1" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A2" s="27"/>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A2" s="19"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
@@ -2491,409 +2383,371 @@
       <c r="F2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="G2" s="23" t="s">
-        <v>240</v>
-      </c>
-      <c r="H2" s="2"/>
-      <c r="I2" s="7"/>
-      <c r="J2" s="23" t="s">
-        <v>239</v>
-      </c>
-      <c r="K2" s="23" t="s">
-        <v>240</v>
-      </c>
-      <c r="L2" s="23" t="s">
-        <v>241</v>
-      </c>
-      <c r="M2" s="23" t="s">
-        <v>240</v>
-      </c>
-      <c r="N2" s="23" t="s">
-        <v>240</v>
-      </c>
-      <c r="O2" s="2"/>
-      <c r="P2" s="2"/>
-      <c r="Q2" s="1"/>
-      <c r="R2" s="1"/>
-    </row>
-    <row r="3" spans="1:18" s="15" customFormat="1" ht="60" x14ac:dyDescent="0.25">
-      <c r="A3" s="28" t="s">
-        <v>182</v>
-      </c>
-      <c r="B3" s="29" t="s">
-        <v>58</v>
-      </c>
-      <c r="C3" s="29" t="s">
-        <v>153</v>
-      </c>
-      <c r="D3" s="29" t="s">
-        <v>41</v>
-      </c>
-      <c r="E3" s="29" t="s">
-        <v>154</v>
-      </c>
-      <c r="F3" s="29" t="s">
-        <v>59</v>
-      </c>
-      <c r="G3" s="24" t="s">
-        <v>155</v>
-      </c>
-      <c r="H3" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="I3" s="29" t="s">
-        <v>156</v>
-      </c>
-      <c r="J3" s="24" t="s">
-        <v>157</v>
-      </c>
-      <c r="K3" s="24" t="s">
-        <v>158</v>
-      </c>
-      <c r="L3" s="24" t="s">
-        <v>10</v>
-      </c>
-      <c r="M3" s="24" t="s">
-        <v>159</v>
-      </c>
-      <c r="N3" s="24" t="s">
-        <v>11</v>
-      </c>
-      <c r="O3" s="29" t="s">
+      <c r="G2" s="2"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
+      <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
+    </row>
+    <row r="3" spans="1:12" s="11" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+      <c r="A3" s="20" t="s">
+        <v>167</v>
+      </c>
+      <c r="B3" s="21" t="s">
+        <v>55</v>
+      </c>
+      <c r="C3" s="21" t="s">
+        <v>150</v>
+      </c>
+      <c r="D3" s="21" t="s">
+        <v>38</v>
+      </c>
+      <c r="E3" s="21" t="s">
+        <v>151</v>
+      </c>
+      <c r="F3" s="21" t="s">
+        <v>56</v>
+      </c>
+      <c r="G3" s="21" t="s">
+        <v>81</v>
+      </c>
+      <c r="H3" s="21" t="s">
+        <v>152</v>
+      </c>
+      <c r="I3" s="21" t="s">
+        <v>19</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="K3" s="21" t="s">
+        <v>18</v>
+      </c>
+      <c r="L3" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="P3" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="Q3" s="29" t="s">
-        <v>20</v>
-      </c>
-      <c r="R3" s="29" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="4" spans="1:18" ht="15.75" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>0</v>
       </c>
       <c r="B4" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C4" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D4" t="str">
         <f t="shared" ref="D4:D12" si="0">_xlfn.CONCAT(B4,":",C4)</f>
         <v>Industrial_roundwood:FI</v>
       </c>
       <c r="E4" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F4">
         <v>0</v>
       </c>
-      <c r="H4" t="s">
-        <v>53</v>
-      </c>
-      <c r="M4" s="4"/>
-      <c r="P4">
+      <c r="G4" t="s">
+        <v>50</v>
+      </c>
+      <c r="J4">
         <v>3.6999999999999998E-2</v>
       </c>
-      <c r="Q4">
+      <c r="K4">
         <v>0.34699999999999998</v>
       </c>
-      <c r="R4" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="5" spans="1:18" ht="15.75" x14ac:dyDescent="0.3">
+      <c r="L4" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D5" t="str">
         <f t="shared" si="0"/>
         <v>Sawmilling:FI</v>
       </c>
       <c r="E5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F5">
         <v>0</v>
       </c>
-      <c r="H5" t="s">
-        <v>53</v>
-      </c>
-      <c r="M5" s="4"/>
-      <c r="P5">
+      <c r="G5" t="s">
+        <v>50</v>
+      </c>
+      <c r="J5">
         <v>0.24299999999999999</v>
       </c>
-      <c r="Q5">
+      <c r="K5">
         <v>0.39200000000000002</v>
       </c>
-      <c r="R5" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="L5" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2</v>
       </c>
       <c r="B6" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C6" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D6" t="str">
         <f t="shared" si="0"/>
         <v>Residues:FI</v>
       </c>
       <c r="E6" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F6">
         <v>0</v>
       </c>
-      <c r="H6" t="s">
-        <v>53</v>
-      </c>
-      <c r="P6">
+      <c r="G6" t="s">
+        <v>50</v>
+      </c>
+      <c r="J6">
         <v>0.40899999999999997</v>
       </c>
-      <c r="Q6">
+      <c r="K6">
         <v>0.05</v>
       </c>
-      <c r="R6" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="L6" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>3</v>
       </c>
       <c r="B7" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C7" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D7" t="str">
         <f t="shared" si="0"/>
         <v>Sawnwood:FI</v>
       </c>
       <c r="E7" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F7">
         <v>0</v>
       </c>
-      <c r="H7" t="s">
-        <v>53</v>
-      </c>
-      <c r="P7">
+      <c r="G7" t="s">
+        <v>50</v>
+      </c>
+      <c r="J7">
         <v>0.40899999999999997</v>
       </c>
-      <c r="Q7">
+      <c r="K7">
         <v>0.53200000000000003</v>
       </c>
-      <c r="R7" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="8" spans="1:18" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L7" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>4</v>
       </c>
       <c r="B8" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C8" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D8" t="str">
         <f t="shared" si="0"/>
         <v>Construction:FI</v>
       </c>
       <c r="E8" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="F8">
         <v>10</v>
       </c>
+      <c r="G8" t="s">
+        <v>35</v>
+      </c>
       <c r="H8" t="s">
-        <v>37</v>
-      </c>
-      <c r="I8" t="s">
-        <v>188</v>
-      </c>
-      <c r="P8">
+        <v>173</v>
+      </c>
+      <c r="J8">
         <v>0.752</v>
       </c>
-      <c r="Q8">
+      <c r="K8">
         <v>0.44400000000000001</v>
       </c>
-      <c r="R8" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="9" spans="1:18" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L8" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>5</v>
       </c>
       <c r="B9" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C9" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D9" t="str">
         <f t="shared" si="0"/>
         <v>Furniture:FI</v>
       </c>
       <c r="E9" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="F9">
         <v>5</v>
       </c>
+      <c r="G9" t="s">
+        <v>35</v>
+      </c>
       <c r="H9" t="s">
-        <v>37</v>
-      </c>
-      <c r="I9" t="s">
-        <v>188</v>
-      </c>
-      <c r="P9">
+        <v>173</v>
+      </c>
+      <c r="J9">
         <v>0.65600000000000003</v>
       </c>
-      <c r="Q9">
+      <c r="K9">
         <v>0.77300000000000002</v>
       </c>
-      <c r="R9" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="L9" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>6</v>
       </c>
       <c r="B10" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C10" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D10" t="str">
         <f t="shared" si="0"/>
         <v>Sawnwood:Import</v>
       </c>
       <c r="E10" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F10">
         <v>0</v>
       </c>
-      <c r="H10" t="s">
-        <v>53</v>
-      </c>
-      <c r="P10">
+      <c r="G10" t="s">
+        <v>50</v>
+      </c>
+      <c r="J10">
         <v>0.24299999999999999</v>
       </c>
-      <c r="Q10">
+      <c r="K10">
         <v>0.9</v>
       </c>
-      <c r="R10" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="L10" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>7</v>
       </c>
       <c r="B11" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C11" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D11" t="str">
         <f t="shared" si="0"/>
         <v>Sawnwood:Export</v>
       </c>
       <c r="E11" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F11">
         <v>0</v>
       </c>
-      <c r="H11" t="s">
-        <v>53</v>
-      </c>
-      <c r="P11">
+      <c r="G11" t="s">
+        <v>50</v>
+      </c>
+      <c r="J11">
         <v>0.69099999999999995</v>
       </c>
-      <c r="Q11">
+      <c r="K11">
         <v>0.16500000000000001</v>
       </c>
-      <c r="R11" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="L11" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>8</v>
       </c>
       <c r="B12" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C12" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D12" t="str">
         <f t="shared" si="0"/>
         <v>Incineration:FI</v>
       </c>
       <c r="E12" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F12">
         <v>0</v>
       </c>
-      <c r="H12" t="s">
-        <v>53</v>
-      </c>
-      <c r="P12">
+      <c r="G12" t="s">
+        <v>50</v>
+      </c>
+      <c r="J12">
         <v>0.96599999999999997</v>
       </c>
-      <c r="Q12">
+      <c r="K12">
         <v>0.48299999999999998</v>
       </c>
-      <c r="R12" t="s">
-        <v>133</v>
+      <c r="L12" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="18" ht="15.6" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <phoneticPr fontId="5" type="noConversion"/>
-  <dataValidations xWindow="1088" yWindow="385" count="2">
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="see parameters.py for more info" prompt="tuple = number or list of parameters separated by comma. Example: stddev=1. For shape and scale list separated by comma e.g., shape=1, scale=1.5_x000a_Normal: stddev_x000a_LogNormal: stddev_x000a_FoldedNormal: stddev_x000a_Weibull: shape, scale_x000a_LandfillDecayWood /Pap: condition_x000a_" sqref="I4:I1048576" xr:uid="{564AD8C3-F96D-40DD-BFD1-1C6E073701B7}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Sankey diagram positioning" prompt="Sankey diagram X and Y node positioning. Check / adjust positioning after you run case and see coordinates. " sqref="Q2 P4:Q1048576" xr:uid="{167D7519-74A2-4731-8D99-C2A980321CC9}"/>
+  <phoneticPr fontId="4" type="noConversion"/>
+  <dataValidations disablePrompts="1" xWindow="1088" yWindow="385" count="2">
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="see parameters.py for more info" prompt="tuple = number or list of parameters separated by comma. Example: stddev=1. For shape and scale list separated by comma e.g., shape=1, scale=1.5_x000a_Normal: stddev_x000a_LogNormal: stddev_x000a_FoldedNormal: stddev_x000a_Weibull: shape, scale_x000a_LandfillDecayWood /Pap: condition_x000a_" sqref="H4:H1048576" xr:uid="{564AD8C3-F96D-40DD-BFD1-1C6E073701B7}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Sankey diagram positioning" prompt="Sankey diagram X and Y node positioning. Check / adjust positioning after you run case and see coordinates. " sqref="K2 J4:K1048576" xr:uid="{167D7519-74A2-4731-8D99-C2A980321CC9}"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" r:id="rId1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xWindow="1088" yWindow="385" count="1">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" disablePrompts="1" xWindow="1088" yWindow="385" count="1">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{DA69398A-0340-441A-BF0A-578EFEF6082C}">
           <x14:formula1>
             <xm:f>'Data validation parameters'!$B$6:$B$14</xm:f>
           </x14:formula1>
-          <xm:sqref>H4:H1048576</xm:sqref>
+          <xm:sqref>G4:G1048576</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -2903,29 +2757,21 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B692AEE8-68EE-4B81-A49D-50BF066DFFE7}">
-  <dimension ref="A1:P91"/>
+  <dimension ref="A1:H91"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.5703125" customWidth="1"/>
-    <col min="2" max="2" width="22" customWidth="1"/>
-    <col min="3" max="3" width="22.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="24.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.7109375" customWidth="1"/>
-    <col min="6" max="6" width="22.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="24" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="24" customWidth="1"/>
-    <col min="9" max="9" width="20.42578125" customWidth="1"/>
-    <col min="10" max="10" width="9.42578125" customWidth="1"/>
-    <col min="11" max="11" width="15.85546875" customWidth="1"/>
-    <col min="12" max="12" width="12.85546875" customWidth="1"/>
-    <col min="13" max="13" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="21.7109375" style="5" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="15.7109375" customWidth="1"/>
-    <col min="16" max="16" width="42" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="3" max="3" width="20.42578125" customWidth="1"/>
+    <col min="4" max="4" width="9.42578125" customWidth="1"/>
+    <col min="5" max="5" width="15.85546875" customWidth="1"/>
+    <col min="6" max="6" width="12.85546875" customWidth="1"/>
+    <col min="7" max="7" width="15.7109375" customWidth="1"/>
+    <col min="8" max="8" width="42" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A1" s="27" t="s">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" s="19" t="s">
         <v>4</v>
       </c>
       <c r="B1" s="2" t="s">
@@ -2935,47 +2781,653 @@
         <v>5</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>5</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>5</v>
       </c>
+    </row>
+    <row r="2" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="H2" s="2"/>
+    </row>
+    <row r="3" spans="1:8" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="20" t="s">
+        <v>168</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>162</v>
+      </c>
+      <c r="H3" s="8" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="D4">
+        <v>60</v>
+      </c>
+      <c r="E4" t="s">
+        <v>39</v>
+      </c>
+      <c r="F4">
+        <v>2021</v>
+      </c>
+      <c r="H4" s="9"/>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>41</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="D5">
+        <v>100</v>
+      </c>
+      <c r="E5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F5">
+        <v>2021</v>
+      </c>
+      <c r="H5" s="9"/>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D6">
+        <v>10</v>
+      </c>
+      <c r="E6" t="s">
+        <v>39</v>
+      </c>
+      <c r="F6">
+        <v>2021</v>
+      </c>
+      <c r="H6" s="9"/>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>47</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="D7">
+        <v>60</v>
+      </c>
+      <c r="E7" t="s">
+        <v>9</v>
+      </c>
+      <c r="F7">
+        <v>2021</v>
+      </c>
+      <c r="G7">
+        <v>0.22500000000000001</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>43</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="D8">
+        <v>40</v>
+      </c>
+      <c r="E8" t="s">
+        <v>9</v>
+      </c>
+      <c r="F8">
+        <v>2021</v>
+      </c>
+      <c r="G8">
+        <v>0.22500000000000001</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>44</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="D9">
+        <v>40</v>
+      </c>
+      <c r="E9" t="s">
+        <v>9</v>
+      </c>
+      <c r="F9">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>45</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="D10">
+        <v>60</v>
+      </c>
+      <c r="E10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F10">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>46</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="D11">
+        <v>100</v>
+      </c>
+      <c r="E11" t="s">
+        <v>9</v>
+      </c>
+      <c r="F11">
+        <v>2021</v>
+      </c>
+      <c r="H11" s="9"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>48</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="D12">
+        <v>20</v>
+      </c>
+      <c r="E12" t="s">
+        <v>39</v>
+      </c>
+      <c r="F12">
+        <v>2021</v>
+      </c>
+      <c r="H12" s="9"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>49</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="D13">
+        <v>10</v>
+      </c>
+      <c r="E13" t="s">
+        <v>39</v>
+      </c>
+      <c r="F13">
+        <v>2021</v>
+      </c>
+      <c r="H13" s="9"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B14" s="3"/>
+      <c r="C14" s="3"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B15" s="3"/>
+      <c r="C15" s="3"/>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B16" s="3"/>
+      <c r="C16" s="3"/>
+    </row>
+    <row r="17" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B17" s="3"/>
+      <c r="C17" s="3"/>
+    </row>
+    <row r="18" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B18" s="3"/>
+      <c r="C18" s="3"/>
+    </row>
+    <row r="19" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B19" s="3"/>
+      <c r="C19" s="3"/>
+    </row>
+    <row r="20" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B20" s="3"/>
+      <c r="C20" s="3"/>
+    </row>
+    <row r="21" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B21" s="3"/>
+      <c r="C21" s="3"/>
+    </row>
+    <row r="22" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B22" s="3"/>
+      <c r="C22" s="3"/>
+    </row>
+    <row r="23" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B23" s="3"/>
+      <c r="C23" s="3"/>
+    </row>
+    <row r="24" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B24" s="3"/>
+      <c r="C24" s="3"/>
+    </row>
+    <row r="25" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B25" s="3"/>
+      <c r="C25" s="3"/>
+    </row>
+    <row r="26" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B26" s="3"/>
+      <c r="C26" s="3"/>
+    </row>
+    <row r="27" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B27" s="3"/>
+      <c r="C27" s="3"/>
+    </row>
+    <row r="28" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B28" s="3"/>
+      <c r="C28" s="3"/>
+    </row>
+    <row r="29" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B29" s="3"/>
+      <c r="C29" s="3"/>
+    </row>
+    <row r="30" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B30" s="3"/>
+      <c r="C30" s="3"/>
+    </row>
+    <row r="31" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B31" s="3"/>
+      <c r="C31" s="3"/>
+    </row>
+    <row r="32" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B32" s="3"/>
+      <c r="C32" s="3"/>
+    </row>
+    <row r="33" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B33" s="3"/>
+      <c r="C33" s="3"/>
+    </row>
+    <row r="34" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B34" s="3"/>
+      <c r="C34" s="3"/>
+    </row>
+    <row r="35" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B35" s="3"/>
+      <c r="C35" s="3"/>
+    </row>
+    <row r="36" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B36" s="3"/>
+      <c r="C36" s="3"/>
+    </row>
+    <row r="37" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B37" s="3"/>
+      <c r="C37" s="3"/>
+    </row>
+    <row r="38" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B38" s="3"/>
+      <c r="C38" s="3"/>
+    </row>
+    <row r="39" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B39" s="3"/>
+      <c r="C39" s="3"/>
+    </row>
+    <row r="40" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B40" s="3"/>
+      <c r="C40" s="3"/>
+    </row>
+    <row r="41" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B41" s="3"/>
+      <c r="C41" s="3"/>
+    </row>
+    <row r="42" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B42" s="3"/>
+      <c r="C42" s="3"/>
+    </row>
+    <row r="43" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B43" s="3"/>
+      <c r="C43" s="3"/>
+    </row>
+    <row r="44" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B44" s="3"/>
+      <c r="C44" s="3"/>
+    </row>
+    <row r="45" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B45" s="3"/>
+      <c r="C45" s="3"/>
+    </row>
+    <row r="46" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B46" s="3"/>
+      <c r="C46" s="3"/>
+    </row>
+    <row r="47" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B47" s="3"/>
+      <c r="C47" s="3"/>
+    </row>
+    <row r="48" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B48" s="3"/>
+      <c r="C48" s="3"/>
+    </row>
+    <row r="49" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B49" s="3"/>
+      <c r="C49" s="3"/>
+    </row>
+    <row r="50" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B50" s="3"/>
+      <c r="C50" s="3"/>
+    </row>
+    <row r="51" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B51" s="3"/>
+      <c r="C51" s="3"/>
+    </row>
+    <row r="52" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B52" s="3"/>
+      <c r="C52" s="3"/>
+    </row>
+    <row r="53" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B53" s="3"/>
+      <c r="C53" s="3"/>
+    </row>
+    <row r="54" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B54" s="3"/>
+      <c r="C54" s="3"/>
+    </row>
+    <row r="55" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B55" s="3"/>
+      <c r="C55" s="3"/>
+    </row>
+    <row r="56" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B56" s="3"/>
+      <c r="C56" s="3"/>
+    </row>
+    <row r="57" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B57" s="3"/>
+      <c r="C57" s="3"/>
+    </row>
+    <row r="58" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B58" s="3"/>
+      <c r="C58" s="3"/>
+    </row>
+    <row r="59" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B59" s="3"/>
+      <c r="C59" s="3"/>
+    </row>
+    <row r="60" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B60" s="3"/>
+      <c r="C60" s="3"/>
+    </row>
+    <row r="61" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B61" s="3"/>
+      <c r="C61" s="3"/>
+    </row>
+    <row r="62" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B62" s="3"/>
+      <c r="C62" s="3"/>
+    </row>
+    <row r="63" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B63" s="3"/>
+      <c r="C63" s="3"/>
+    </row>
+    <row r="64" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B64" s="3"/>
+      <c r="C64" s="3"/>
+    </row>
+    <row r="65" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B65" s="3"/>
+      <c r="C65" s="3"/>
+    </row>
+    <row r="66" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B66" s="3"/>
+      <c r="C66" s="3"/>
+    </row>
+    <row r="67" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B67" s="3"/>
+      <c r="C67" s="3"/>
+    </row>
+    <row r="68" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B68" s="3"/>
+      <c r="C68" s="3"/>
+    </row>
+    <row r="69" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B69" s="3"/>
+      <c r="C69" s="3"/>
+    </row>
+    <row r="70" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B70" s="3"/>
+      <c r="C70" s="3"/>
+    </row>
+    <row r="71" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B71" s="3"/>
+      <c r="C71" s="3"/>
+    </row>
+    <row r="72" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B72" s="3"/>
+      <c r="C72" s="3"/>
+    </row>
+    <row r="73" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B73" s="3"/>
+      <c r="C73" s="3"/>
+    </row>
+    <row r="74" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B74" s="3"/>
+      <c r="C74" s="3"/>
+    </row>
+    <row r="75" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B75" s="3"/>
+      <c r="C75" s="3"/>
+    </row>
+    <row r="76" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B76" s="3"/>
+      <c r="C76" s="3"/>
+    </row>
+    <row r="77" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B77" s="3"/>
+      <c r="C77" s="3"/>
+    </row>
+    <row r="78" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B78" s="3"/>
+      <c r="C78" s="3"/>
+    </row>
+    <row r="79" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B79" s="3"/>
+      <c r="C79" s="3"/>
+    </row>
+    <row r="80" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B80" s="3"/>
+      <c r="C80" s="3"/>
+    </row>
+    <row r="81" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B81" s="3"/>
+      <c r="C81" s="3"/>
+    </row>
+    <row r="82" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B82" s="3"/>
+      <c r="C82" s="3"/>
+    </row>
+    <row r="83" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B83" s="3"/>
+      <c r="C83" s="3"/>
+    </row>
+    <row r="84" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B84" s="3"/>
+      <c r="C84" s="3"/>
+    </row>
+    <row r="85" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B85" s="3"/>
+      <c r="C85" s="3"/>
+    </row>
+    <row r="87" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B87" s="3"/>
+      <c r="C87" s="3"/>
+    </row>
+    <row r="88" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B88" s="3"/>
+      <c r="C88" s="3"/>
+    </row>
+    <row r="89" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B89" s="3"/>
+      <c r="C89" s="3"/>
+    </row>
+    <row r="90" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B90" s="3"/>
+      <c r="C90" s="3"/>
+    </row>
+    <row r="91" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B91" s="3"/>
+      <c r="C91" s="3"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A3:H13" xr:uid="{B692AEE8-68EE-4B81-A49D-50BF066DFFE7}"/>
+  <phoneticPr fontId="4" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{29AEC29D-2905-49D6-A378-57F89A2CFFA2}">
+          <x14:formula1>
+            <xm:f>Processes!$D$4:$D$1048576</xm:f>
+          </x14:formula1>
+          <xm:sqref>B4:C13</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD427C93-5971-4A1F-9BA5-0A112F61A8DE}">
+  <dimension ref="A1:J4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="37.85546875" customWidth="1"/>
+    <col min="2" max="2" width="23.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="8" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="35.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A1" s="19" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>199</v>
+      </c>
       <c r="I1" s="2" t="s">
         <v>5</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="K1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="M1" s="23" t="s">
-        <v>5</v>
-      </c>
-      <c r="N1" s="23" t="s">
-        <v>5</v>
-      </c>
-      <c r="O1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="P1" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="27" t="s">
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" s="19" t="s">
         <v>8</v>
       </c>
       <c r="B2" s="2"/>
@@ -2987,1014 +3439,37 @@
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
       <c r="J2" s="2"/>
-      <c r="K2" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="L2" s="2"/>
-      <c r="M2" s="23" t="s">
-        <v>240</v>
-      </c>
-      <c r="N2" s="23" t="s">
-        <v>240</v>
-      </c>
-      <c r="O2" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="P2" s="2"/>
-    </row>
-    <row r="3" spans="1:16" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="28" t="s">
-        <v>183</v>
-      </c>
-      <c r="B3" s="9" t="s">
-        <v>164</v>
-      </c>
-      <c r="C3" s="9" t="s">
-        <v>154</v>
-      </c>
-      <c r="D3" s="9" t="s">
-        <v>165</v>
-      </c>
-      <c r="E3" s="9" t="s">
-        <v>166</v>
-      </c>
-      <c r="F3" s="9" t="s">
-        <v>154</v>
-      </c>
-      <c r="G3" s="9" t="s">
-        <v>167</v>
-      </c>
-      <c r="H3" s="9" t="s">
-        <v>168</v>
-      </c>
-      <c r="I3" s="9" t="s">
-        <v>169</v>
-      </c>
-      <c r="J3" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="K3" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="L3" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="M3" s="25" t="s">
-        <v>170</v>
-      </c>
-      <c r="N3" s="26" t="s">
-        <v>171</v>
-      </c>
-      <c r="O3" s="11" t="s">
-        <v>177</v>
-      </c>
-      <c r="P3" s="12" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>43</v>
-      </c>
-      <c r="B4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C4" t="str">
-        <f>+_xlfn.XLOOKUP(H4,Processes!$D$4:$D$47,Processes!$E$4:$E$47)</f>
-        <v>Source</v>
-      </c>
-      <c r="D4" t="s">
-        <v>26</v>
-      </c>
-      <c r="E4" t="s">
-        <v>29</v>
-      </c>
-      <c r="F4" t="str">
-        <f>+_xlfn.XLOOKUP(I4,Processes!$D$4:$D$47,Processes!$E$4:$E$47)</f>
-        <v>First</v>
-      </c>
-      <c r="G4" t="s">
-        <v>26</v>
-      </c>
-      <c r="H4" s="3" t="str">
-        <f t="shared" ref="H4:H13" si="0">_xlfn.CONCAT(B4,":",D4)</f>
-        <v>Industrial_roundwood:FI</v>
-      </c>
-      <c r="I4" s="3" t="str">
-        <f t="shared" ref="I4:I13" si="1">_xlfn.CONCAT(E4,":",G4)</f>
-        <v>Sawmilling:FI</v>
-      </c>
-      <c r="J4">
-        <v>60</v>
-      </c>
-      <c r="K4" t="s">
-        <v>42</v>
-      </c>
-      <c r="L4">
-        <v>2021</v>
-      </c>
-      <c r="N4" t="s">
+    </row>
+    <row r="3" spans="1:10" ht="60.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="20" t="s">
+        <v>200</v>
+      </c>
+      <c r="B3" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="P4" s="13"/>
-    </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>44</v>
-      </c>
-      <c r="B5" t="s">
-        <v>29</v>
-      </c>
-      <c r="C5" t="str">
-        <f>+_xlfn.XLOOKUP(H5,Processes!$D$4:$D$47,Processes!$E$4:$E$47)</f>
-        <v>First</v>
-      </c>
-      <c r="D5" t="s">
-        <v>26</v>
-      </c>
-      <c r="E5" t="s">
-        <v>28</v>
-      </c>
-      <c r="F5" t="str">
-        <f>+_xlfn.XLOOKUP(I5,Processes!$D$4:$D$47,Processes!$E$4:$E$47)</f>
-        <v>Second</v>
-      </c>
-      <c r="G5" t="s">
-        <v>26</v>
-      </c>
-      <c r="H5" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>Sawmilling:FI</v>
-      </c>
-      <c r="I5" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>Sawnwood:FI</v>
-      </c>
-      <c r="J5">
-        <v>100</v>
-      </c>
-      <c r="K5" t="s">
-        <v>9</v>
-      </c>
-      <c r="L5">
-        <v>2021</v>
-      </c>
-      <c r="N5" t="s">
-        <v>38</v>
-      </c>
-      <c r="P5" s="13"/>
-    </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>45</v>
-      </c>
-      <c r="B6" t="s">
-        <v>29</v>
-      </c>
-      <c r="C6" t="str">
-        <f>+_xlfn.XLOOKUP(H6,Processes!$D$4:$D$47,Processes!$E$4:$E$47)</f>
-        <v>First</v>
-      </c>
-      <c r="D6" t="s">
-        <v>26</v>
-      </c>
-      <c r="E6" t="s">
-        <v>32</v>
-      </c>
-      <c r="F6" t="str">
-        <f>+_xlfn.XLOOKUP(I6,Processes!$D$4:$D$47,Processes!$E$4:$E$47)</f>
-        <v>by_prod</v>
-      </c>
-      <c r="G6" t="s">
-        <v>26</v>
-      </c>
-      <c r="H6" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>Sawmilling:FI</v>
-      </c>
-      <c r="I6" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>Residues:FI</v>
-      </c>
-      <c r="J6">
+      <c r="C3" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>201</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="I3" s="6" t="s">
+        <v>204</v>
+      </c>
+      <c r="J3" s="5" t="s">
         <v>10</v>
-      </c>
-      <c r="K6" t="s">
-        <v>42</v>
-      </c>
-      <c r="L6">
-        <v>2021</v>
-      </c>
-      <c r="N6" t="s">
-        <v>38</v>
-      </c>
-      <c r="P6" s="13"/>
-    </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>50</v>
-      </c>
-      <c r="B7" t="s">
-        <v>28</v>
-      </c>
-      <c r="C7" t="str">
-        <f>+_xlfn.XLOOKUP(H7,Processes!$D$4:$D$47,Processes!$E$4:$E$47)</f>
-        <v>Second</v>
-      </c>
-      <c r="D7" t="s">
-        <v>26</v>
-      </c>
-      <c r="E7" t="s">
-        <v>30</v>
-      </c>
-      <c r="F7" t="str">
-        <f>+_xlfn.XLOOKUP(I7,Processes!$D$4:$D$47,Processes!$E$4:$E$47)</f>
-        <v>VAM</v>
-      </c>
-      <c r="G7" t="s">
-        <v>26</v>
-      </c>
-      <c r="H7" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>Sawnwood:FI</v>
-      </c>
-      <c r="I7" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>Construction:FI</v>
-      </c>
-      <c r="J7">
-        <v>60</v>
-      </c>
-      <c r="K7" t="s">
-        <v>9</v>
-      </c>
-      <c r="L7">
-        <v>2021</v>
-      </c>
-      <c r="N7" t="s">
-        <v>38</v>
-      </c>
-      <c r="O7">
-        <v>0.22500000000000001</v>
-      </c>
-    </row>
-    <row r="8" spans="1:16" ht="18.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>46</v>
-      </c>
-      <c r="B8" t="s">
-        <v>28</v>
-      </c>
-      <c r="C8" t="str">
-        <f>+_xlfn.XLOOKUP(H8,Processes!$D$4:$D$47,Processes!$E$4:$E$47)</f>
-        <v>Second</v>
-      </c>
-      <c r="D8" t="s">
-        <v>26</v>
-      </c>
-      <c r="E8" t="s">
-        <v>31</v>
-      </c>
-      <c r="F8" t="str">
-        <f>+_xlfn.XLOOKUP(I8,Processes!$D$4:$D$47,Processes!$E$4:$E$47)</f>
-        <v>VAM</v>
-      </c>
-      <c r="G8" t="s">
-        <v>26</v>
-      </c>
-      <c r="H8" s="3" t="str">
-        <f>_xlfn.CONCAT(B8,":",D8)</f>
-        <v>Sawnwood:FI</v>
-      </c>
-      <c r="I8" s="3" t="str">
-        <f>_xlfn.CONCAT(E8,":",G8)</f>
-        <v>Furniture:FI</v>
-      </c>
-      <c r="J8">
-        <v>40</v>
-      </c>
-      <c r="K8" t="s">
-        <v>9</v>
-      </c>
-      <c r="L8">
-        <v>2021</v>
-      </c>
-      <c r="N8" t="s">
-        <v>38</v>
-      </c>
-      <c r="O8">
-        <v>0.22500000000000001</v>
-      </c>
-    </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>47</v>
-      </c>
-      <c r="B9" t="s">
-        <v>30</v>
-      </c>
-      <c r="C9" t="str">
-        <f>+_xlfn.XLOOKUP(H9,Processes!$D$4:$D$47,Processes!$E$4:$E$47)</f>
-        <v>VAM</v>
-      </c>
-      <c r="D9" t="s">
-        <v>26</v>
-      </c>
-      <c r="E9" t="s">
-        <v>29</v>
-      </c>
-      <c r="F9" t="str">
-        <f>+_xlfn.XLOOKUP(I9,Processes!$D$4:$D$47,Processes!$E$4:$E$47)</f>
-        <v>First</v>
-      </c>
-      <c r="G9" t="s">
-        <v>26</v>
-      </c>
-      <c r="H9" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>Construction:FI</v>
-      </c>
-      <c r="I9" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>Sawmilling:FI</v>
-      </c>
-      <c r="J9">
-        <v>40</v>
-      </c>
-      <c r="K9" t="s">
-        <v>9</v>
-      </c>
-      <c r="L9">
-        <v>2021</v>
-      </c>
-      <c r="N9" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="10" spans="1:16" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>48</v>
-      </c>
-      <c r="B10" t="s">
-        <v>30</v>
-      </c>
-      <c r="C10" t="str">
-        <f>+_xlfn.XLOOKUP(H10,Processes!$D$4:$D$47,Processes!$E$4:$E$47)</f>
-        <v>VAM</v>
-      </c>
-      <c r="D10" t="s">
-        <v>26</v>
-      </c>
-      <c r="E10" t="s">
-        <v>33</v>
-      </c>
-      <c r="F10" t="str">
-        <f>+_xlfn.XLOOKUP(I10,Processes!$D$4:$D$47,Processes!$E$4:$E$47)</f>
-        <v>EoL</v>
-      </c>
-      <c r="G10" t="s">
-        <v>26</v>
-      </c>
-      <c r="H10" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>Construction:FI</v>
-      </c>
-      <c r="I10" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>Incineration:FI</v>
-      </c>
-      <c r="J10">
-        <v>60</v>
-      </c>
-      <c r="K10" t="s">
-        <v>9</v>
-      </c>
-      <c r="L10">
-        <v>2021</v>
-      </c>
-      <c r="N10" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>49</v>
-      </c>
-      <c r="B11" t="s">
-        <v>31</v>
-      </c>
-      <c r="C11" t="s">
-        <v>36</v>
-      </c>
-      <c r="D11" t="s">
-        <v>26</v>
-      </c>
-      <c r="E11" t="s">
-        <v>33</v>
-      </c>
-      <c r="F11" t="str">
-        <f>+_xlfn.XLOOKUP(I11,Processes!$D$4:$D$47,Processes!$E$4:$E$47)</f>
-        <v>EoL</v>
-      </c>
-      <c r="G11" t="s">
-        <v>26</v>
-      </c>
-      <c r="H11" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>Furniture:FI</v>
-      </c>
-      <c r="I11" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>Incineration:FI</v>
-      </c>
-      <c r="J11">
-        <v>100</v>
-      </c>
-      <c r="K11" t="s">
-        <v>9</v>
-      </c>
-      <c r="L11">
-        <v>2021</v>
-      </c>
-      <c r="N11" t="s">
-        <v>38</v>
-      </c>
-      <c r="P11" s="13"/>
-    </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>51</v>
-      </c>
-      <c r="B12" t="s">
-        <v>28</v>
-      </c>
-      <c r="C12" t="str">
-        <f>+_xlfn.XLOOKUP(H12,Processes!$D$4:$D$47,Processes!$E$4:$E$47)</f>
-        <v>Second</v>
-      </c>
-      <c r="D12" t="s">
-        <v>26</v>
-      </c>
-      <c r="E12" t="s">
-        <v>28</v>
-      </c>
-      <c r="F12" t="str">
-        <f>+_xlfn.XLOOKUP(I12,Processes!$D$4:$D$47,Processes!$E$4:$E$47)</f>
-        <v>RoW</v>
-      </c>
-      <c r="G12" t="s">
-        <v>18</v>
-      </c>
-      <c r="H12" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>Sawnwood:FI</v>
-      </c>
-      <c r="I12" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>Sawnwood:Export</v>
-      </c>
-      <c r="J12">
-        <v>20</v>
-      </c>
-      <c r="K12" t="s">
-        <v>42</v>
-      </c>
-      <c r="L12">
-        <v>2021</v>
-      </c>
-      <c r="N12" t="s">
-        <v>38</v>
-      </c>
-      <c r="P12" s="13"/>
-    </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>52</v>
-      </c>
-      <c r="B13" t="s">
-        <v>28</v>
-      </c>
-      <c r="C13" t="str">
-        <f>+_xlfn.XLOOKUP(H13,Processes!$D$4:$D$47,Processes!$E$4:$E$47)</f>
-        <v>RoW</v>
-      </c>
-      <c r="D13" t="s">
-        <v>17</v>
-      </c>
-      <c r="E13" t="s">
-        <v>28</v>
-      </c>
-      <c r="F13" t="str">
-        <f>+_xlfn.XLOOKUP(I13,Processes!$D$4:$D$47,Processes!$E$4:$E$47)</f>
-        <v>Second</v>
-      </c>
-      <c r="G13" t="s">
-        <v>26</v>
-      </c>
-      <c r="H13" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>Sawnwood:Import</v>
-      </c>
-      <c r="I13" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>Sawnwood:FI</v>
-      </c>
-      <c r="J13">
-        <v>10</v>
-      </c>
-      <c r="K13" t="s">
-        <v>42</v>
-      </c>
-      <c r="L13">
-        <v>2021</v>
-      </c>
-      <c r="N13" t="s">
-        <v>38</v>
-      </c>
-      <c r="P13" s="13"/>
-    </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="H14" s="3"/>
-      <c r="I14" s="3"/>
-      <c r="N14"/>
-    </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="H15" s="3"/>
-      <c r="I15" s="3"/>
-      <c r="N15"/>
-    </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="H16" s="3"/>
-      <c r="I16" s="3"/>
-      <c r="N16"/>
-    </row>
-    <row r="17" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H17" s="3"/>
-      <c r="I17" s="3"/>
-      <c r="N17"/>
-    </row>
-    <row r="18" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H18" s="3"/>
-      <c r="I18" s="3"/>
-      <c r="N18"/>
-    </row>
-    <row r="19" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H19" s="3"/>
-      <c r="I19" s="3"/>
-      <c r="N19"/>
-    </row>
-    <row r="20" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H20" s="3"/>
-      <c r="I20" s="3"/>
-      <c r="N20"/>
-    </row>
-    <row r="21" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H21" s="3"/>
-      <c r="I21" s="3"/>
-      <c r="N21"/>
-    </row>
-    <row r="22" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H22" s="3"/>
-      <c r="I22" s="3"/>
-      <c r="N22"/>
-    </row>
-    <row r="23" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H23" s="3"/>
-      <c r="I23" s="3"/>
-      <c r="N23"/>
-    </row>
-    <row r="24" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H24" s="3"/>
-      <c r="I24" s="3"/>
-    </row>
-    <row r="25" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H25" s="3"/>
-      <c r="I25" s="3"/>
-    </row>
-    <row r="26" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H26" s="3"/>
-      <c r="I26" s="3"/>
-    </row>
-    <row r="27" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H27" s="3"/>
-      <c r="I27" s="3"/>
-    </row>
-    <row r="28" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H28" s="3"/>
-      <c r="I28" s="3"/>
-      <c r="N28" s="6"/>
-    </row>
-    <row r="29" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H29" s="3"/>
-      <c r="I29" s="3"/>
-      <c r="N29" s="6"/>
-    </row>
-    <row r="30" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H30" s="3"/>
-      <c r="I30" s="3"/>
-    </row>
-    <row r="31" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H31" s="3"/>
-      <c r="I31" s="3"/>
-    </row>
-    <row r="32" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H32" s="3"/>
-      <c r="I32" s="3"/>
-    </row>
-    <row r="33" spans="3:14" x14ac:dyDescent="0.25">
-      <c r="H33" s="3"/>
-      <c r="I33" s="3"/>
-    </row>
-    <row r="34" spans="3:14" x14ac:dyDescent="0.25">
-      <c r="H34" s="3"/>
-      <c r="I34" s="3"/>
-    </row>
-    <row r="35" spans="3:14" x14ac:dyDescent="0.25">
-      <c r="E35" s="13"/>
-      <c r="H35" s="3"/>
-      <c r="I35" s="3"/>
-    </row>
-    <row r="36" spans="3:14" x14ac:dyDescent="0.25">
-      <c r="H36" s="3"/>
-      <c r="I36" s="3"/>
-    </row>
-    <row r="37" spans="3:14" x14ac:dyDescent="0.25">
-      <c r="H37" s="3"/>
-      <c r="I37" s="3"/>
-    </row>
-    <row r="38" spans="3:14" x14ac:dyDescent="0.25">
-      <c r="H38" s="3"/>
-      <c r="I38" s="3"/>
-    </row>
-    <row r="39" spans="3:14" x14ac:dyDescent="0.25">
-      <c r="H39" s="3"/>
-      <c r="I39" s="3"/>
-      <c r="N39"/>
-    </row>
-    <row r="40" spans="3:14" x14ac:dyDescent="0.25">
-      <c r="H40" s="3"/>
-      <c r="I40" s="3"/>
-      <c r="N40"/>
-    </row>
-    <row r="41" spans="3:14" x14ac:dyDescent="0.25">
-      <c r="H41" s="3"/>
-      <c r="I41" s="3"/>
-      <c r="N41"/>
-    </row>
-    <row r="42" spans="3:14" x14ac:dyDescent="0.25">
-      <c r="H42" s="3"/>
-      <c r="I42" s="3"/>
-      <c r="N42"/>
-    </row>
-    <row r="43" spans="3:14" x14ac:dyDescent="0.25">
-      <c r="H43" s="3"/>
-      <c r="I43" s="3"/>
-      <c r="N43"/>
-    </row>
-    <row r="44" spans="3:14" x14ac:dyDescent="0.25">
-      <c r="H44" s="3"/>
-      <c r="I44" s="3"/>
-      <c r="N44"/>
-    </row>
-    <row r="45" spans="3:14" x14ac:dyDescent="0.25">
-      <c r="C45" s="8"/>
-      <c r="H45" s="3"/>
-      <c r="I45" s="3"/>
-      <c r="N45"/>
-    </row>
-    <row r="46" spans="3:14" x14ac:dyDescent="0.25">
-      <c r="H46" s="3"/>
-      <c r="I46" s="3"/>
-      <c r="N46"/>
-    </row>
-    <row r="47" spans="3:14" x14ac:dyDescent="0.25">
-      <c r="H47" s="3"/>
-      <c r="I47" s="3"/>
-      <c r="N47"/>
-    </row>
-    <row r="48" spans="3:14" x14ac:dyDescent="0.25">
-      <c r="H48" s="3"/>
-      <c r="I48" s="3"/>
-      <c r="N48"/>
-    </row>
-    <row r="49" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H49" s="3"/>
-      <c r="I49" s="3"/>
-      <c r="N49"/>
-    </row>
-    <row r="50" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H50" s="3"/>
-      <c r="I50" s="3"/>
-      <c r="N50"/>
-    </row>
-    <row r="51" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H51" s="3"/>
-      <c r="I51" s="3"/>
-      <c r="N51"/>
-    </row>
-    <row r="52" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H52" s="3"/>
-      <c r="I52" s="3"/>
-      <c r="N52"/>
-    </row>
-    <row r="53" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H53" s="3"/>
-      <c r="I53" s="3"/>
-      <c r="N53"/>
-    </row>
-    <row r="54" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H54" s="3"/>
-      <c r="I54" s="3"/>
-      <c r="N54"/>
-    </row>
-    <row r="55" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H55" s="3"/>
-      <c r="I55" s="3"/>
-      <c r="N55"/>
-    </row>
-    <row r="56" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H56" s="3"/>
-      <c r="I56" s="3"/>
-      <c r="N56"/>
-    </row>
-    <row r="57" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H57" s="3"/>
-      <c r="I57" s="3"/>
-      <c r="N57"/>
-    </row>
-    <row r="58" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H58" s="3"/>
-      <c r="I58" s="3"/>
-      <c r="N58"/>
-    </row>
-    <row r="59" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H59" s="3"/>
-      <c r="I59" s="3"/>
-      <c r="N59"/>
-    </row>
-    <row r="60" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H60" s="3"/>
-      <c r="I60" s="3"/>
-      <c r="N60"/>
-    </row>
-    <row r="61" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H61" s="3"/>
-      <c r="I61" s="3"/>
-      <c r="N61"/>
-    </row>
-    <row r="62" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H62" s="3"/>
-      <c r="I62" s="3"/>
-      <c r="N62"/>
-    </row>
-    <row r="63" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H63" s="3"/>
-      <c r="I63" s="3"/>
-      <c r="N63"/>
-    </row>
-    <row r="64" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H64" s="3"/>
-      <c r="I64" s="3"/>
-      <c r="N64"/>
-    </row>
-    <row r="65" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H65" s="3"/>
-      <c r="I65" s="3"/>
-      <c r="N65"/>
-    </row>
-    <row r="66" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H66" s="3"/>
-      <c r="I66" s="3"/>
-      <c r="N66"/>
-    </row>
-    <row r="67" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H67" s="3"/>
-      <c r="I67" s="3"/>
-      <c r="N67"/>
-    </row>
-    <row r="68" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H68" s="3"/>
-      <c r="I68" s="3"/>
-      <c r="N68"/>
-    </row>
-    <row r="69" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H69" s="3"/>
-      <c r="I69" s="3"/>
-      <c r="N69"/>
-    </row>
-    <row r="70" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H70" s="3"/>
-      <c r="I70" s="3"/>
-      <c r="N70"/>
-    </row>
-    <row r="71" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H71" s="3"/>
-      <c r="I71" s="3"/>
-      <c r="N71"/>
-    </row>
-    <row r="72" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H72" s="3"/>
-      <c r="I72" s="3"/>
-      <c r="N72"/>
-    </row>
-    <row r="73" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H73" s="3"/>
-      <c r="I73" s="3"/>
-      <c r="N73"/>
-    </row>
-    <row r="74" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H74" s="3"/>
-      <c r="I74" s="3"/>
-      <c r="N74"/>
-    </row>
-    <row r="75" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H75" s="3"/>
-      <c r="I75" s="3"/>
-      <c r="N75"/>
-    </row>
-    <row r="76" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H76" s="3"/>
-      <c r="I76" s="3"/>
-      <c r="N76"/>
-    </row>
-    <row r="77" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H77" s="3"/>
-      <c r="I77" s="3"/>
-      <c r="N77"/>
-    </row>
-    <row r="78" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H78" s="3"/>
-      <c r="I78" s="3"/>
-      <c r="N78"/>
-    </row>
-    <row r="79" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H79" s="3"/>
-      <c r="I79" s="3"/>
-      <c r="N79"/>
-    </row>
-    <row r="80" spans="8:14" x14ac:dyDescent="0.25">
-      <c r="H80" s="3"/>
-      <c r="I80" s="3"/>
-      <c r="N80"/>
-    </row>
-    <row r="81" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="H81" s="3"/>
-      <c r="I81" s="3"/>
-      <c r="N81"/>
-    </row>
-    <row r="82" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="H82" s="3"/>
-      <c r="I82" s="3"/>
-      <c r="N82"/>
-    </row>
-    <row r="83" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="H83" s="3"/>
-      <c r="I83" s="3"/>
-      <c r="N83"/>
-    </row>
-    <row r="84" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="H84" s="3"/>
-      <c r="I84" s="3"/>
-      <c r="N84"/>
-    </row>
-    <row r="85" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="H85" s="3"/>
-      <c r="I85" s="3"/>
-      <c r="N85"/>
-    </row>
-    <row r="86" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="N86"/>
-    </row>
-    <row r="87" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B87" s="3"/>
-      <c r="D87" s="3"/>
-      <c r="E87" s="3"/>
-      <c r="G87" s="3"/>
-      <c r="H87" s="3"/>
-      <c r="I87" s="3"/>
-      <c r="M87" s="3"/>
-      <c r="N87"/>
-    </row>
-    <row r="88" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="H88" s="3"/>
-      <c r="I88" s="3"/>
-      <c r="N88"/>
-    </row>
-    <row r="89" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="H89" s="3"/>
-      <c r="I89" s="3"/>
-      <c r="N89"/>
-    </row>
-    <row r="90" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="H90" s="3"/>
-      <c r="I90" s="3"/>
-      <c r="N90"/>
-    </row>
-    <row r="91" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="H91" s="3"/>
-      <c r="I91" s="3"/>
-      <c r="N91"/>
-    </row>
-  </sheetData>
-  <autoFilter ref="A3:P13" xr:uid="{B692AEE8-68EE-4B81-A49D-50BF066DFFE7}"/>
-  <phoneticPr fontId="5" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-  <drawing r:id="rId2"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD427C93-5971-4A1F-9BA5-0A112F61A8DE}">
-  <dimension ref="A1:J4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="37.85546875" customWidth="1"/>
-    <col min="2" max="2" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="8" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="35.7109375" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A1" s="27" t="s">
-        <v>4</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>214</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>214</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>214</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="27" t="s">
-        <v>8</v>
-      </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
-    </row>
-    <row r="3" spans="1:10" ht="60.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="28" t="s">
-        <v>215</v>
-      </c>
-      <c r="B3" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="C3" s="9" t="s">
-        <v>59</v>
-      </c>
-      <c r="D3" s="9" t="s">
-        <v>110</v>
-      </c>
-      <c r="E3" s="9" t="s">
-        <v>111</v>
-      </c>
-      <c r="F3" s="9" t="s">
-        <v>216</v>
-      </c>
-      <c r="G3" s="9" t="s">
-        <v>217</v>
-      </c>
-      <c r="H3" s="9" t="s">
-        <v>218</v>
-      </c>
-      <c r="I3" s="10" t="s">
-        <v>219</v>
-      </c>
-      <c r="J3" s="9" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
@@ -4002,19 +3477,25 @@
     </row>
   </sheetData>
   <dataValidations xWindow="985" yWindow="379" count="3">
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="NOTE" prompt="Used only in the following stock distribution types:_x000a_- Normal_x000a_- LogNormal_x000a_- FoldedNormal" sqref="F4:F1048576 F3" xr:uid="{EB58ED90-11CC-40D7-B560-63144E99B293}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="NOTE" prompt="Used only in the following stock distribution types:_x000a_- Weibull" sqref="G3:G1048576 H3:H4 H6:H1048576 H5" xr:uid="{C2A4F33A-4C0F-44AA-B773-8DCE440EA2FB}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="NOTE" prompt="Used only in the following stock distribution types:_x000a_- Normal_x000a_- LogNormal_x000a_- FoldedNormal" sqref="F3:F1048576" xr:uid="{EB58ED90-11CC-40D7-B560-63144E99B293}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="NOTE" prompt="Used only in the following stock distribution types:_x000a_- Weibull" sqref="G3:H1048576" xr:uid="{C2A4F33A-4C0F-44AA-B773-8DCE440EA2FB}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="NOTE" prompt="Used only in the following stock distribution types:_x000a_- LandfillDecayWood_x000a_- LandfillDecayPaper" sqref="I3" xr:uid="{9247F767-8020-484B-8E5F-041BF9D0E8CE}"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xWindow="985" yWindow="379" count="1">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xWindow="985" yWindow="379" count="2">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="NOTE" prompt="Used only in the following stock distribution types:_x000a_- LandfillDecayWood_x000a_- LandfillDecayPaper" xr:uid="{23BA98F2-1DDD-4331-B721-E5AC9432C3B0}">
           <x14:formula1>
             <xm:f>'Data validation parameters'!$H$6:$H$9</xm:f>
           </x14:formula1>
-          <xm:sqref>I5:I1048576 I4</xm:sqref>
+          <xm:sqref>I4:I1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{C60080E3-0027-44EC-8134-4F98E88A9910}">
+          <x14:formula1>
+            <xm:f>Processes!$D$4:$D$12</xm:f>
+          </x14:formula1>
+          <xm:sqref>B5:B1048576</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -4034,17 +3515,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="B1" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="C1" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="D1" s="9" t="s">
-        <v>20</v>
+      <c r="A1" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -4052,7 +3533,7 @@
         <v>2021</v>
       </c>
       <c r="B2" t="s">
-        <v>201</v>
+        <v>186</v>
       </c>
       <c r="C2">
         <v>3.6999999999999998E-2</v>
@@ -4066,7 +3547,7 @@
         <v>2021</v>
       </c>
       <c r="B3" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C3">
         <v>0.24299999999999999</v>
@@ -4080,7 +3561,7 @@
         <v>2021</v>
       </c>
       <c r="B4" t="s">
-        <v>202</v>
+        <v>187</v>
       </c>
       <c r="C4">
         <v>0.40899999999999997</v>
@@ -4094,7 +3575,7 @@
         <v>2021</v>
       </c>
       <c r="B5" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C5">
         <v>0.40899999999999997</v>
@@ -4108,7 +3589,7 @@
         <v>2021</v>
       </c>
       <c r="B6" t="s">
-        <v>203</v>
+        <v>188</v>
       </c>
       <c r="C6">
         <v>0.752</v>
@@ -4122,7 +3603,7 @@
         <v>2021</v>
       </c>
       <c r="B7" t="s">
-        <v>204</v>
+        <v>189</v>
       </c>
       <c r="C7">
         <v>0.65600000000000003</v>
@@ -4136,7 +3617,7 @@
         <v>2021</v>
       </c>
       <c r="B8" t="s">
-        <v>205</v>
+        <v>190</v>
       </c>
       <c r="C8">
         <v>0.96599999999999997</v>
@@ -4150,7 +3631,7 @@
         <v>2021</v>
       </c>
       <c r="B9" t="s">
-        <v>206</v>
+        <v>191</v>
       </c>
       <c r="C9">
         <v>0.69099999999999995</v>
@@ -4164,7 +3645,7 @@
         <v>2021</v>
       </c>
       <c r="B10" t="s">
-        <v>207</v>
+        <v>192</v>
       </c>
       <c r="C10">
         <v>0.24299999999999999</v>
@@ -4178,7 +3659,7 @@
         <v>2022</v>
       </c>
       <c r="B11" t="s">
-        <v>201</v>
+        <v>186</v>
       </c>
       <c r="C11">
         <v>3.6999999999999998E-2</v>
@@ -4192,7 +3673,7 @@
         <v>2022</v>
       </c>
       <c r="B12" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C12">
         <v>0.24299999999999999</v>
@@ -4206,7 +3687,7 @@
         <v>2022</v>
       </c>
       <c r="B13" t="s">
-        <v>202</v>
+        <v>187</v>
       </c>
       <c r="C13">
         <v>0.40899999999999997</v>
@@ -4220,7 +3701,7 @@
         <v>2022</v>
       </c>
       <c r="B14" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C14">
         <v>0.40899999999999997</v>
@@ -4234,7 +3715,7 @@
         <v>2022</v>
       </c>
       <c r="B15" t="s">
-        <v>203</v>
+        <v>188</v>
       </c>
       <c r="C15">
         <v>0.752</v>
@@ -4248,7 +3729,7 @@
         <v>2022</v>
       </c>
       <c r="B16" t="s">
-        <v>204</v>
+        <v>189</v>
       </c>
       <c r="C16">
         <v>0.65600000000000003</v>
@@ -4262,7 +3743,7 @@
         <v>2022</v>
       </c>
       <c r="B17" t="s">
-        <v>205</v>
+        <v>190</v>
       </c>
       <c r="C17">
         <v>0.96599999999999997</v>
@@ -4276,7 +3757,7 @@
         <v>2022</v>
       </c>
       <c r="B18" t="s">
-        <v>206</v>
+        <v>191</v>
       </c>
       <c r="C18">
         <v>0.69099999999999995</v>
@@ -4290,7 +3771,7 @@
         <v>2022</v>
       </c>
       <c r="B19" t="s">
-        <v>207</v>
+        <v>192</v>
       </c>
       <c r="C19">
         <v>0.24299999999999999</v>
@@ -4304,7 +3785,7 @@
         <v>2023</v>
       </c>
       <c r="B20" t="s">
-        <v>201</v>
+        <v>186</v>
       </c>
       <c r="C20">
         <v>3.6999999999999998E-2</v>
@@ -4318,7 +3799,7 @@
         <v>2023</v>
       </c>
       <c r="B21" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C21">
         <v>0.24299999999999999</v>
@@ -4332,7 +3813,7 @@
         <v>2023</v>
       </c>
       <c r="B22" t="s">
-        <v>202</v>
+        <v>187</v>
       </c>
       <c r="C22">
         <v>0.40899999999999997</v>
@@ -4346,7 +3827,7 @@
         <v>2023</v>
       </c>
       <c r="B23" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C23">
         <v>0.40899999999999997</v>
@@ -4360,7 +3841,7 @@
         <v>2023</v>
       </c>
       <c r="B24" t="s">
-        <v>203</v>
+        <v>188</v>
       </c>
       <c r="C24">
         <v>0.752</v>
@@ -4374,7 +3855,7 @@
         <v>2023</v>
       </c>
       <c r="B25" t="s">
-        <v>204</v>
+        <v>189</v>
       </c>
       <c r="C25">
         <v>0.65600000000000003</v>
@@ -4388,7 +3869,7 @@
         <v>2023</v>
       </c>
       <c r="B26" t="s">
-        <v>205</v>
+        <v>190</v>
       </c>
       <c r="C26">
         <v>0.96599999999999997</v>
@@ -4402,7 +3883,7 @@
         <v>2023</v>
       </c>
       <c r="B27" t="s">
-        <v>206</v>
+        <v>191</v>
       </c>
       <c r="C27">
         <v>0.69099999999999995</v>
@@ -4416,7 +3897,7 @@
         <v>2023</v>
       </c>
       <c r="B28" t="s">
-        <v>207</v>
+        <v>192</v>
       </c>
       <c r="C28">
         <v>0.24299999999999999</v>
@@ -4430,7 +3911,7 @@
         <v>2024</v>
       </c>
       <c r="B29" t="s">
-        <v>201</v>
+        <v>186</v>
       </c>
       <c r="C29">
         <v>3.6999999999999998E-2</v>
@@ -4444,7 +3925,7 @@
         <v>2024</v>
       </c>
       <c r="B30" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C30">
         <v>0.24299999999999999</v>
@@ -4458,7 +3939,7 @@
         <v>2024</v>
       </c>
       <c r="B31" t="s">
-        <v>202</v>
+        <v>187</v>
       </c>
       <c r="C31">
         <v>0.40899999999999997</v>
@@ -4472,7 +3953,7 @@
         <v>2024</v>
       </c>
       <c r="B32" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C32">
         <v>0.40899999999999997</v>
@@ -4486,7 +3967,7 @@
         <v>2024</v>
       </c>
       <c r="B33" t="s">
-        <v>203</v>
+        <v>188</v>
       </c>
       <c r="C33">
         <v>0.752</v>
@@ -4500,7 +3981,7 @@
         <v>2024</v>
       </c>
       <c r="B34" t="s">
-        <v>204</v>
+        <v>189</v>
       </c>
       <c r="C34">
         <v>0.65600000000000003</v>
@@ -4514,7 +3995,7 @@
         <v>2024</v>
       </c>
       <c r="B35" t="s">
-        <v>205</v>
+        <v>190</v>
       </c>
       <c r="C35">
         <v>0.96599999999999997</v>
@@ -4528,7 +4009,7 @@
         <v>2024</v>
       </c>
       <c r="B36" t="s">
-        <v>206</v>
+        <v>191</v>
       </c>
       <c r="C36">
         <v>0.69099999999999995</v>
@@ -4542,7 +4023,7 @@
         <v>2024</v>
       </c>
       <c r="B37" t="s">
-        <v>207</v>
+        <v>192</v>
       </c>
       <c r="C37">
         <v>0.24299999999999999</v>
@@ -4556,7 +4037,7 @@
         <v>2025</v>
       </c>
       <c r="B38" t="s">
-        <v>201</v>
+        <v>186</v>
       </c>
       <c r="C38">
         <v>3.6999999999999998E-2</v>
@@ -4570,7 +4051,7 @@
         <v>2025</v>
       </c>
       <c r="B39" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C39">
         <v>0.24299999999999999</v>
@@ -4584,7 +4065,7 @@
         <v>2025</v>
       </c>
       <c r="B40" t="s">
-        <v>202</v>
+        <v>187</v>
       </c>
       <c r="C40">
         <v>0.40899999999999997</v>
@@ -4598,7 +4079,7 @@
         <v>2025</v>
       </c>
       <c r="B41" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C41">
         <v>0.40899999999999997</v>
@@ -4612,7 +4093,7 @@
         <v>2025</v>
       </c>
       <c r="B42" t="s">
-        <v>203</v>
+        <v>188</v>
       </c>
       <c r="C42">
         <v>0.752</v>
@@ -4626,7 +4107,7 @@
         <v>2025</v>
       </c>
       <c r="B43" t="s">
-        <v>204</v>
+        <v>189</v>
       </c>
       <c r="C43">
         <v>0.65600000000000003</v>
@@ -4640,7 +4121,7 @@
         <v>2025</v>
       </c>
       <c r="B44" t="s">
-        <v>205</v>
+        <v>190</v>
       </c>
       <c r="C44">
         <v>0.96599999999999997</v>
@@ -4654,7 +4135,7 @@
         <v>2025</v>
       </c>
       <c r="B45" t="s">
-        <v>206</v>
+        <v>191</v>
       </c>
       <c r="C45">
         <v>0.69099999999999995</v>
@@ -4668,7 +4149,7 @@
         <v>2025</v>
       </c>
       <c r="B46" t="s">
-        <v>207</v>
+        <v>192</v>
       </c>
       <c r="C46">
         <v>0.24299999999999999</v>
@@ -4682,7 +4163,7 @@
         <v>2026</v>
       </c>
       <c r="B47" t="s">
-        <v>201</v>
+        <v>186</v>
       </c>
       <c r="C47">
         <v>3.6999999999999998E-2</v>
@@ -4696,7 +4177,7 @@
         <v>2026</v>
       </c>
       <c r="B48" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C48">
         <v>0.24299999999999999</v>
@@ -4710,7 +4191,7 @@
         <v>2026</v>
       </c>
       <c r="B49" t="s">
-        <v>202</v>
+        <v>187</v>
       </c>
       <c r="C49">
         <v>0.40899999999999997</v>
@@ -4724,7 +4205,7 @@
         <v>2026</v>
       </c>
       <c r="B50" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C50">
         <v>0.40899999999999997</v>
@@ -4738,7 +4219,7 @@
         <v>2026</v>
       </c>
       <c r="B51" t="s">
-        <v>203</v>
+        <v>188</v>
       </c>
       <c r="C51">
         <v>0.752</v>
@@ -4752,7 +4233,7 @@
         <v>2026</v>
       </c>
       <c r="B52" t="s">
-        <v>204</v>
+        <v>189</v>
       </c>
       <c r="C52">
         <v>0.65600000000000003</v>
@@ -4766,7 +4247,7 @@
         <v>2026</v>
       </c>
       <c r="B53" t="s">
-        <v>205</v>
+        <v>190</v>
       </c>
       <c r="C53">
         <v>0.96599999999999997</v>
@@ -4780,7 +4261,7 @@
         <v>2026</v>
       </c>
       <c r="B54" t="s">
-        <v>206</v>
+        <v>191</v>
       </c>
       <c r="C54">
         <v>0.69099999999999995</v>
@@ -4794,7 +4275,7 @@
         <v>2026</v>
       </c>
       <c r="B55" t="s">
-        <v>207</v>
+        <v>192</v>
       </c>
       <c r="C55">
         <v>0.24299999999999999</v>
@@ -4808,7 +4289,7 @@
         <v>2027</v>
       </c>
       <c r="B56" t="s">
-        <v>201</v>
+        <v>186</v>
       </c>
       <c r="C56">
         <v>3.6999999999999998E-2</v>
@@ -4822,7 +4303,7 @@
         <v>2027</v>
       </c>
       <c r="B57" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C57">
         <v>0.24299999999999999</v>
@@ -4836,7 +4317,7 @@
         <v>2027</v>
       </c>
       <c r="B58" t="s">
-        <v>202</v>
+        <v>187</v>
       </c>
       <c r="C58">
         <v>0.40899999999999997</v>
@@ -4850,7 +4331,7 @@
         <v>2027</v>
       </c>
       <c r="B59" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C59">
         <v>0.40899999999999997</v>
@@ -4864,7 +4345,7 @@
         <v>2027</v>
       </c>
       <c r="B60" t="s">
-        <v>203</v>
+        <v>188</v>
       </c>
       <c r="C60">
         <v>0.752</v>
@@ -4878,7 +4359,7 @@
         <v>2027</v>
       </c>
       <c r="B61" t="s">
-        <v>204</v>
+        <v>189</v>
       </c>
       <c r="C61">
         <v>0.65600000000000003</v>
@@ -4892,7 +4373,7 @@
         <v>2027</v>
       </c>
       <c r="B62" t="s">
-        <v>205</v>
+        <v>190</v>
       </c>
       <c r="C62">
         <v>0.96599999999999997</v>
@@ -4906,7 +4387,7 @@
         <v>2027</v>
       </c>
       <c r="B63" t="s">
-        <v>206</v>
+        <v>191</v>
       </c>
       <c r="C63">
         <v>0.69099999999999995</v>
@@ -4920,7 +4401,7 @@
         <v>2027</v>
       </c>
       <c r="B64" t="s">
-        <v>207</v>
+        <v>192</v>
       </c>
       <c r="C64">
         <v>0.24299999999999999</v>
@@ -4934,7 +4415,7 @@
         <v>2028</v>
       </c>
       <c r="B65" t="s">
-        <v>201</v>
+        <v>186</v>
       </c>
       <c r="C65">
         <v>3.6999999999999998E-2</v>
@@ -4948,7 +4429,7 @@
         <v>2028</v>
       </c>
       <c r="B66" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C66">
         <v>0.24299999999999999</v>
@@ -4962,7 +4443,7 @@
         <v>2028</v>
       </c>
       <c r="B67" t="s">
-        <v>202</v>
+        <v>187</v>
       </c>
       <c r="C67">
         <v>0.40899999999999997</v>
@@ -4976,7 +4457,7 @@
         <v>2028</v>
       </c>
       <c r="B68" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C68">
         <v>0.40899999999999997</v>
@@ -4990,7 +4471,7 @@
         <v>2028</v>
       </c>
       <c r="B69" t="s">
-        <v>203</v>
+        <v>188</v>
       </c>
       <c r="C69">
         <v>0.752</v>
@@ -5004,7 +4485,7 @@
         <v>2028</v>
       </c>
       <c r="B70" t="s">
-        <v>204</v>
+        <v>189</v>
       </c>
       <c r="C70">
         <v>0.65600000000000003</v>
@@ -5018,7 +4499,7 @@
         <v>2028</v>
       </c>
       <c r="B71" t="s">
-        <v>205</v>
+        <v>190</v>
       </c>
       <c r="C71">
         <v>0.96599999999999997</v>
@@ -5032,7 +4513,7 @@
         <v>2028</v>
       </c>
       <c r="B72" t="s">
-        <v>206</v>
+        <v>191</v>
       </c>
       <c r="C72">
         <v>0.69099999999999995</v>
@@ -5046,7 +4527,7 @@
         <v>2028</v>
       </c>
       <c r="B73" t="s">
-        <v>207</v>
+        <v>192</v>
       </c>
       <c r="C73">
         <v>0.24299999999999999</v>
@@ -5060,7 +4541,7 @@
         <v>2029</v>
       </c>
       <c r="B74" t="s">
-        <v>201</v>
+        <v>186</v>
       </c>
       <c r="C74">
         <v>3.6999999999999998E-2</v>
@@ -5074,7 +4555,7 @@
         <v>2029</v>
       </c>
       <c r="B75" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C75">
         <v>0.24299999999999999</v>
@@ -5088,7 +4569,7 @@
         <v>2029</v>
       </c>
       <c r="B76" t="s">
-        <v>202</v>
+        <v>187</v>
       </c>
       <c r="C76">
         <v>0.40899999999999997</v>
@@ -5102,7 +4583,7 @@
         <v>2029</v>
       </c>
       <c r="B77" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C77">
         <v>0.40899999999999997</v>
@@ -5116,7 +4597,7 @@
         <v>2029</v>
       </c>
       <c r="B78" t="s">
-        <v>203</v>
+        <v>188</v>
       </c>
       <c r="C78">
         <v>0.752</v>
@@ -5130,7 +4611,7 @@
         <v>2029</v>
       </c>
       <c r="B79" t="s">
-        <v>204</v>
+        <v>189</v>
       </c>
       <c r="C79">
         <v>0.65600000000000003</v>
@@ -5144,7 +4625,7 @@
         <v>2029</v>
       </c>
       <c r="B80" t="s">
-        <v>205</v>
+        <v>190</v>
       </c>
       <c r="C80">
         <v>0.96599999999999997</v>
@@ -5158,7 +4639,7 @@
         <v>2029</v>
       </c>
       <c r="B81" t="s">
-        <v>206</v>
+        <v>191</v>
       </c>
       <c r="C81">
         <v>0.69099999999999995</v>
@@ -5172,7 +4653,7 @@
         <v>2029</v>
       </c>
       <c r="B82" t="s">
-        <v>207</v>
+        <v>192</v>
       </c>
       <c r="C82">
         <v>0.24299999999999999</v>
@@ -5186,7 +4667,7 @@
         <v>2030</v>
       </c>
       <c r="B83" t="s">
-        <v>201</v>
+        <v>186</v>
       </c>
       <c r="C83">
         <v>3.6999999999999998E-2</v>
@@ -5200,7 +4681,7 @@
         <v>2030</v>
       </c>
       <c r="B84" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C84">
         <v>0.24299999999999999</v>
@@ -5214,7 +4695,7 @@
         <v>2030</v>
       </c>
       <c r="B85" t="s">
-        <v>202</v>
+        <v>187</v>
       </c>
       <c r="C85">
         <v>0.40899999999999997</v>
@@ -5228,7 +4709,7 @@
         <v>2030</v>
       </c>
       <c r="B86" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C86">
         <v>0.40899999999999997</v>
@@ -5242,7 +4723,7 @@
         <v>2030</v>
       </c>
       <c r="B87" t="s">
-        <v>203</v>
+        <v>188</v>
       </c>
       <c r="C87">
         <v>0.752</v>
@@ -5256,7 +4737,7 @@
         <v>2030</v>
       </c>
       <c r="B88" t="s">
-        <v>204</v>
+        <v>189</v>
       </c>
       <c r="C88">
         <v>0.65600000000000003</v>
@@ -5270,7 +4751,7 @@
         <v>2030</v>
       </c>
       <c r="B89" t="s">
-        <v>205</v>
+        <v>190</v>
       </c>
       <c r="C89">
         <v>0.96599999999999997</v>
@@ -5284,7 +4765,7 @@
         <v>2030</v>
       </c>
       <c r="B90" t="s">
-        <v>206</v>
+        <v>191</v>
       </c>
       <c r="C90">
         <v>0.69099999999999995</v>
@@ -5298,7 +4779,7 @@
         <v>2030</v>
       </c>
       <c r="B91" t="s">
-        <v>207</v>
+        <v>192</v>
       </c>
       <c r="C91">
         <v>0.24299999999999999</v>
@@ -5333,56 +4814,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A1" s="27"/>
-      <c r="B1" s="30" t="s">
+      <c r="A1" s="19"/>
+      <c r="B1" s="22" t="s">
+        <v>102</v>
+      </c>
+      <c r="C1" s="22" t="s">
+        <v>103</v>
+      </c>
+      <c r="D1" s="22" t="s">
+        <v>104</v>
+      </c>
+      <c r="E1" s="22" t="s">
         <v>105</v>
       </c>
-      <c r="C1" s="30" t="s">
+      <c r="F1" s="22" t="s">
+        <v>171</v>
+      </c>
+      <c r="G1" s="22" t="s">
         <v>106</v>
       </c>
-      <c r="D1" s="30" t="s">
+      <c r="H1" s="22" t="s">
         <v>107</v>
       </c>
-      <c r="E1" s="30" t="s">
+      <c r="I1" s="22" t="s">
         <v>108</v>
       </c>
-      <c r="F1" s="30" t="s">
-        <v>186</v>
-      </c>
-      <c r="G1" s="30" t="s">
+      <c r="J1" s="22" t="s">
         <v>109</v>
       </c>
-      <c r="H1" s="30" t="s">
+      <c r="K1" s="22" t="s">
+        <v>193</v>
+      </c>
+      <c r="L1" s="22" t="s">
         <v>110</v>
       </c>
-      <c r="I1" s="30" t="s">
-        <v>111</v>
-      </c>
-      <c r="J1" s="30" t="s">
-        <v>112</v>
-      </c>
-      <c r="K1" s="30" t="s">
-        <v>208</v>
-      </c>
-      <c r="L1" s="30" t="s">
-        <v>113</v>
-      </c>
-      <c r="M1" s="30" t="s">
-        <v>113</v>
+      <c r="M1" s="22" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="2" spans="1:13" ht="30" x14ac:dyDescent="0.25">
-      <c r="A2" s="28" t="s">
-        <v>245</v>
+      <c r="A2" s="20" t="s">
+        <v>225</v>
       </c>
       <c r="B2" t="s">
-        <v>179</v>
+        <v>164</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="E2">
         <v>-50</v>
@@ -5397,9 +4878,9 @@
         <v>2030</v>
       </c>
       <c r="J2" t="s">
-        <v>119</v>
-      </c>
-      <c r="K2" s="22" t="b">
+        <v>116</v>
+      </c>
+      <c r="K2" s="18" t="b">
         <v>1</v>
       </c>
     </row>
@@ -5420,7 +4901,7 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{283A9876-07D1-4356-BD7B-618A4AD94BB4}">
           <x14:formula1>
             <xm:f>'Data validation parameters'!$F$6:$F$9</xm:f>
@@ -5432,6 +4913,12 @@
             <xm:f>'Data validation parameters'!$E$6:$E$7</xm:f>
           </x14:formula1>
           <xm:sqref>G2 F1:F2 F5:F1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{EE0A79EA-3499-4925-8C21-DDB578FC1E2B}">
+          <x14:formula1>
+            <xm:f>Processes!$D$4:$D$1048576</xm:f>
+          </x14:formula1>
+          <xm:sqref>C2:D1048576</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -5449,78 +4936,78 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="9" t="s">
-        <v>135</v>
-      </c>
-      <c r="B1" s="9" t="s">
-        <v>136</v>
+      <c r="A1" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B4" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B5" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B6" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B7" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B8" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="B9" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="C9" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
     </row>
   </sheetData>
@@ -5546,126 +5033,126 @@
   <sheetData>
     <row r="2" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
     </row>
     <row r="3" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
     </row>
     <row r="5" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B5" s="16" t="s">
-        <v>84</v>
-      </c>
-      <c r="C5" s="16" t="s">
-        <v>72</v>
-      </c>
-      <c r="D5" s="16" t="s">
-        <v>93</v>
-      </c>
-      <c r="E5" s="16" t="s">
-        <v>117</v>
-      </c>
-      <c r="F5" s="16" t="s">
-        <v>112</v>
-      </c>
-      <c r="G5" s="16" t="s">
-        <v>194</v>
-      </c>
-      <c r="H5" s="16" t="s">
-        <v>220</v>
+      <c r="B5" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="D5" s="12" t="s">
+        <v>90</v>
+      </c>
+      <c r="E5" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="F5" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="G5" s="12" t="s">
+        <v>179</v>
+      </c>
+      <c r="H5" s="12" t="s">
+        <v>205</v>
       </c>
     </row>
     <row r="6" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="C6" t="b">
         <v>1</v>
       </c>
       <c r="D6" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="E6" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="F6" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="G6" t="s">
-        <v>195</v>
+        <v>180</v>
       </c>
       <c r="H6" t="s">
-        <v>221</v>
+        <v>206</v>
       </c>
     </row>
     <row r="7" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C7" t="b">
         <v>0</v>
       </c>
       <c r="D7" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="E7" t="s">
         <v>9</v>
       </c>
       <c r="F7" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="G7" t="s">
-        <v>196</v>
+        <v>181</v>
       </c>
       <c r="H7" t="s">
-        <v>222</v>
+        <v>207</v>
       </c>
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="D8" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="F8" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="H8" t="s">
-        <v>223</v>
+        <v>208</v>
       </c>
     </row>
     <row r="9" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="D9" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="F9" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="10" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
     </row>
     <row r="11" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="12" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
-        <v>191</v>
+        <v>176</v>
       </c>
     </row>
     <row r="13" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
-        <v>192</v>
+        <v>177</v>
       </c>
     </row>
   </sheetData>

</xml_diff>